<commit_message>
All Project : Add Coverage To Summary
</commit_message>
<xml_diff>
--- a/GeneticAlgorithm/summary.xlsx
+++ b/GeneticAlgorithm/summary.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rd8e2d7b4748b45e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="2" r:id="R0cb1dd058bd74b9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc446afe663a547ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="2" r:id="R254b849b0ffc469a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="3" r:id="R78f077a05cae4169"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,11 +15,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="3">
     <x:numFmt numFmtId="200" formatCode="0.00"/>
     <x:numFmt numFmtId="201" formatCode="#,##0"/>
+    <x:numFmt numFmtId="202" formatCode="0.00%"/>
   </x:numFmts>
-  <x:fonts count="8">
+  <x:fonts count="13">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -61,8 +63,37 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Aptos"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:color rgb="FF18263B"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF18263B"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FF18263B"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF18263B"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -84,6 +115,16 @@
         <x:fgColor rgb="FF246A73"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF172B49"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF172B49"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -91,7 +132,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="21">
+  <x:cellXfs count="32">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -113,6 +154,25 @@
     <x:xf numFmtId="201" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -336,12 +396,13 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="19" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="19" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="29" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="23" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="23" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -357,7 +418,7 @@
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="4" t="str">
-        <x:v>Round 1 and Round 2 · 851 targets each</x:v>
+        <x:v>Saved V2 results from Round1 and Round2</x:v>
       </x:c>
       <x:c r="B2" s="4"/>
       <x:c r="C2" s="4"/>
@@ -391,7 +452,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="9" t="str">
-        <x:v>Round 1</x:v>
+        <x:v>Round1</x:v>
       </x:c>
       <x:c r="B5" s="15" t="n">
         <x:v>851</x:v>
@@ -406,15 +467,15 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="F5" s="10" t="n">
-        <x:v>53.76</x:v>
+        <x:v>53.76321384425218</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>61.43</x:v>
+        <x:v>61.42649446494468</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="9" t="str">
-        <x:v>Round 2</x:v>
+        <x:v>Round2</x:v>
       </x:c>
       <x:c r="B6" s="15" t="n">
         <x:v>851</x:v>
@@ -429,10 +490,10 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="F6" s="10" t="n">
-        <x:v>54.06</x:v>
+        <x:v>54.06117503059977</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>61.66</x:v>
+        <x:v>61.664141291108436</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -479,7 +540,7 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="8" t="str">
-        <x:v>Chart · R1</x:v>
+        <x:v>Chart / Round1</x:v>
       </x:c>
       <x:c r="B10" s="19" t="n">
         <x:v>26</x:v>
@@ -494,15 +555,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F10" s="14" t="n">
-        <x:v>70.53</x:v>
+        <x:v>70.5304</x:v>
       </x:c>
       <x:c r="G10" s="14" t="n">
-        <x:v>77.9</x:v>
+        <x:v>77.9023076923077</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="8" t="str">
-        <x:v>Chart · R2</x:v>
+        <x:v>Chart / Round2</x:v>
       </x:c>
       <x:c r="B11" s="19" t="n">
         <x:v>26</x:v>
@@ -517,15 +578,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F11" s="14" t="n">
-        <x:v>70.53</x:v>
+        <x:v>70.5304</x:v>
       </x:c>
       <x:c r="G11" s="14" t="n">
-        <x:v>77.9</x:v>
+        <x:v>77.9023076923077</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="8" t="str">
-        <x:v>Cli · R1</x:v>
+        <x:v>Cli / Round1</x:v>
       </x:c>
       <x:c r="B12" s="19" t="n">
         <x:v>39</x:v>
@@ -540,15 +601,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F12" s="14" t="n">
-        <x:v>12.04</x:v>
+        <x:v>12.038205128205128</x:v>
       </x:c>
       <x:c r="G12" s="14" t="n">
-        <x:v>13.4</x:v>
+        <x:v>13.39897435897436</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="8" t="str">
-        <x:v>Cli · R2</x:v>
+        <x:v>Cli / Round2</x:v>
       </x:c>
       <x:c r="B13" s="19" t="n">
         <x:v>39</x:v>
@@ -563,15 +624,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F13" s="14" t="n">
-        <x:v>12.04</x:v>
+        <x:v>12.038205128205128</x:v>
       </x:c>
       <x:c r="G13" s="14" t="n">
-        <x:v>13.4</x:v>
+        <x:v>13.39897435897436</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="8" t="str">
-        <x:v>Closure · R1</x:v>
+        <x:v>Closure / Round1</x:v>
       </x:c>
       <x:c r="B14" s="19" t="n">
         <x:v>174</x:v>
@@ -586,15 +647,15 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="F14" s="14" t="n">
-        <x:v>20.51</x:v>
+        <x:v>20.511972789115642</x:v>
       </x:c>
       <x:c r="G14" s="14" t="n">
-        <x:v>31.97</x:v>
+        <x:v>31.966054421768696</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="8" t="str">
-        <x:v>Closure · R2</x:v>
+        <x:v>Closure / Round2</x:v>
       </x:c>
       <x:c r="B15" s="19" t="n">
         <x:v>174</x:v>
@@ -609,15 +670,15 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="F15" s="14" t="n">
-        <x:v>20.51</x:v>
+        <x:v>20.511972789115642</x:v>
       </x:c>
       <x:c r="G15" s="14" t="n">
-        <x:v>31.97</x:v>
+        <x:v>31.966054421768696</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="8" t="str">
-        <x:v>Codec · R1</x:v>
+        <x:v>Codec / Round1</x:v>
       </x:c>
       <x:c r="B16" s="19" t="n">
         <x:v>18</x:v>
@@ -632,15 +693,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F16" s="14" t="n">
-        <x:v>83.67</x:v>
+        <x:v>83.67444444444445</x:v>
       </x:c>
       <x:c r="G16" s="14" t="n">
-        <x:v>87.87</x:v>
+        <x:v>87.86888888888889</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="8" t="str">
-        <x:v>Codec · R2</x:v>
+        <x:v>Codec / Round2</x:v>
       </x:c>
       <x:c r="B17" s="19" t="n">
         <x:v>18</x:v>
@@ -655,15 +716,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F17" s="14" t="n">
-        <x:v>83.67</x:v>
+        <x:v>83.67444444444445</x:v>
       </x:c>
       <x:c r="G17" s="14" t="n">
-        <x:v>87.87</x:v>
+        <x:v>87.86888888888889</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="8" t="str">
-        <x:v>Collections · R1</x:v>
+        <x:v>Collections / Round1</x:v>
       </x:c>
       <x:c r="B18" s="19" t="n">
         <x:v>28</x:v>
@@ -678,15 +739,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F18" s="14" t="n">
-        <x:v>79.24</x:v>
+        <x:v>79.24071428571429</x:v>
       </x:c>
       <x:c r="G18" s="14" t="n">
-        <x:v>80.45</x:v>
+        <x:v>80.44571428571429</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="8" t="str">
-        <x:v>Collections · R2</x:v>
+        <x:v>Collections / Round2</x:v>
       </x:c>
       <x:c r="B19" s="19" t="n">
         <x:v>28</x:v>
@@ -701,15 +762,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F19" s="14" t="n">
-        <x:v>79.24</x:v>
+        <x:v>79.24071428571429</x:v>
       </x:c>
       <x:c r="G19" s="14" t="n">
-        <x:v>80.45</x:v>
+        <x:v>80.44571428571429</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="8" t="str">
-        <x:v>Compress · R1</x:v>
+        <x:v>Compress / Round1</x:v>
       </x:c>
       <x:c r="B20" s="19" t="n">
         <x:v>47</x:v>
@@ -724,15 +785,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F20" s="14" t="n">
-        <x:v>62.06</x:v>
+        <x:v>62.05872340425531</x:v>
       </x:c>
       <x:c r="G20" s="14" t="n">
-        <x:v>66.19</x:v>
+        <x:v>66.18999999999998</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="8" t="str">
-        <x:v>Compress · R2</x:v>
+        <x:v>Compress / Round2</x:v>
       </x:c>
       <x:c r="B21" s="19" t="n">
         <x:v>47</x:v>
@@ -747,15 +808,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F21" s="14" t="n">
-        <x:v>62.06</x:v>
+        <x:v>62.05872340425531</x:v>
       </x:c>
       <x:c r="G21" s="14" t="n">
-        <x:v>66.19</x:v>
+        <x:v>66.18999999999998</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="8" t="str">
-        <x:v>Csv · R1</x:v>
+        <x:v>Csv / Round1</x:v>
       </x:c>
       <x:c r="B22" s="19" t="n">
         <x:v>16</x:v>
@@ -770,15 +831,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F22" s="14" t="n">
-        <x:v>79.79</x:v>
+        <x:v>79.791875</x:v>
       </x:c>
       <x:c r="G22" s="14" t="n">
-        <x:v>87.8</x:v>
+        <x:v>87.80000000000001</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="8" t="str">
-        <x:v>Csv · R2</x:v>
+        <x:v>Csv / Round2</x:v>
       </x:c>
       <x:c r="B23" s="19" t="n">
         <x:v>16</x:v>
@@ -793,15 +854,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F23" s="14" t="n">
-        <x:v>79.79</x:v>
+        <x:v>79.791875</x:v>
       </x:c>
       <x:c r="G23" s="14" t="n">
-        <x:v>87.8</x:v>
+        <x:v>87.80000000000001</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="8" t="str">
-        <x:v>Gson · R1</x:v>
+        <x:v>Gson / Round1</x:v>
       </x:c>
       <x:c r="B24" s="19" t="n">
         <x:v>17</x:v>
@@ -816,15 +877,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F24" s="14" t="n">
-        <x:v>34.98</x:v>
+        <x:v>34.98117647058824</x:v>
       </x:c>
       <x:c r="G24" s="14" t="n">
-        <x:v>42.28</x:v>
+        <x:v>42.284705882352945</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="8" t="str">
-        <x:v>Gson · R2</x:v>
+        <x:v>Gson / Round2</x:v>
       </x:c>
       <x:c r="B25" s="19" t="n">
         <x:v>17</x:v>
@@ -839,15 +900,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F25" s="14" t="n">
-        <x:v>34.98</x:v>
+        <x:v>34.98117647058824</x:v>
       </x:c>
       <x:c r="G25" s="14" t="n">
-        <x:v>42.28</x:v>
+        <x:v>42.284705882352945</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="8" t="str">
-        <x:v>JacksonCore · R1</x:v>
+        <x:v>JacksonCore / Round1</x:v>
       </x:c>
       <x:c r="B26" s="19" t="n">
         <x:v>24</x:v>
@@ -862,15 +923,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F26" s="14" t="n">
-        <x:v>47.09</x:v>
+        <x:v>47.09125</x:v>
       </x:c>
       <x:c r="G26" s="14" t="n">
-        <x:v>56.5</x:v>
+        <x:v>56.49958333333334</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="8" t="str">
-        <x:v>JacksonCore · R2</x:v>
+        <x:v>JacksonCore / Round2</x:v>
       </x:c>
       <x:c r="B27" s="19" t="n">
         <x:v>24</x:v>
@@ -885,15 +946,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F27" s="14" t="n">
-        <x:v>47.09</x:v>
+        <x:v>47.09125</x:v>
       </x:c>
       <x:c r="G27" s="14" t="n">
-        <x:v>56.5</x:v>
+        <x:v>56.49958333333334</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="8" t="str">
-        <x:v>JacksonDatabind · R1</x:v>
+        <x:v>JacksonDatabind / Round1</x:v>
       </x:c>
       <x:c r="B28" s="19" t="n">
         <x:v>110</x:v>
@@ -908,15 +969,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F28" s="14" t="n">
-        <x:v>47.47</x:v>
+        <x:v>47.46763636363637</x:v>
       </x:c>
       <x:c r="G28" s="14" t="n">
-        <x:v>59.08</x:v>
+        <x:v>59.077909090909095</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="8" t="str">
-        <x:v>JacksonDatabind · R2</x:v>
+        <x:v>JacksonDatabind / Round2</x:v>
       </x:c>
       <x:c r="B29" s="19" t="n">
         <x:v>110</x:v>
@@ -931,15 +992,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F29" s="14" t="n">
-        <x:v>47.47</x:v>
+        <x:v>47.46763636363637</x:v>
       </x:c>
       <x:c r="G29" s="14" t="n">
-        <x:v>59.08</x:v>
+        <x:v>59.077909090909095</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="8" t="str">
-        <x:v>JacksonXml · R1</x:v>
+        <x:v>JacksonXml / Round1</x:v>
       </x:c>
       <x:c r="B30" s="19" t="n">
         <x:v>6</x:v>
@@ -954,15 +1015,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F30" s="14" t="n">
-        <x:v>24.13</x:v>
+        <x:v>24.133333333333336</x:v>
       </x:c>
       <x:c r="G30" s="14" t="n">
-        <x:v>30.19</x:v>
+        <x:v>30.191666666666674</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="8" t="str">
-        <x:v>JacksonXml · R2</x:v>
+        <x:v>JacksonXml / Round2</x:v>
       </x:c>
       <x:c r="B31" s="19" t="n">
         <x:v>6</x:v>
@@ -977,15 +1038,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F31" s="14" t="n">
-        <x:v>24.13</x:v>
+        <x:v>24.133333333333336</x:v>
       </x:c>
       <x:c r="G31" s="14" t="n">
-        <x:v>30.19</x:v>
+        <x:v>30.191666666666674</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="8" t="str">
-        <x:v>Jsoup · R1</x:v>
+        <x:v>Jsoup / Round1</x:v>
       </x:c>
       <x:c r="B32" s="19" t="n">
         <x:v>93</x:v>
@@ -1000,15 +1061,15 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="F32" s="14" t="n">
-        <x:v>61.55</x:v>
+        <x:v>61.55322222222221</x:v>
       </x:c>
       <x:c r="G32" s="14" t="n">
-        <x:v>68.99</x:v>
+        <x:v>68.99055555555555</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="8" t="str">
-        <x:v>Jsoup · R2</x:v>
+        <x:v>Jsoup / Round2</x:v>
       </x:c>
       <x:c r="B33" s="19" t="n">
         <x:v>93</x:v>
@@ -1023,15 +1084,15 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="F33" s="14" t="n">
-        <x:v>61.55</x:v>
+        <x:v>61.55322222222221</x:v>
       </x:c>
       <x:c r="G33" s="14" t="n">
-        <x:v>68.99</x:v>
+        <x:v>68.99055555555555</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="8" t="str">
-        <x:v>JxPath · R1</x:v>
+        <x:v>JxPath / Round1</x:v>
       </x:c>
       <x:c r="B34" s="19" t="n">
         <x:v>22</x:v>
@@ -1046,15 +1107,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F34" s="14" t="n">
-        <x:v>71.15</x:v>
+        <x:v>71.1490909090909</x:v>
       </x:c>
       <x:c r="G34" s="14" t="n">
-        <x:v>78.35</x:v>
+        <x:v>78.3490909090909</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="8" t="str">
-        <x:v>JxPath · R2</x:v>
+        <x:v>JxPath / Round2</x:v>
       </x:c>
       <x:c r="B35" s="19" t="n">
         <x:v>22</x:v>
@@ -1069,15 +1130,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F35" s="14" t="n">
-        <x:v>71.15</x:v>
+        <x:v>71.1490909090909</x:v>
       </x:c>
       <x:c r="G35" s="14" t="n">
-        <x:v>78.35</x:v>
+        <x:v>78.3490909090909</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="8" t="str">
-        <x:v>Lang · R1</x:v>
+        <x:v>Lang / Round1</x:v>
       </x:c>
       <x:c r="B36" s="19" t="n">
         <x:v>61</x:v>
@@ -1092,15 +1153,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F36" s="14" t="n">
-        <x:v>79.33</x:v>
+        <x:v>79.32803278688525</x:v>
       </x:c>
       <x:c r="G36" s="14" t="n">
-        <x:v>84.32</x:v>
+        <x:v>84.32409836065574</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="8" t="str">
-        <x:v>Lang · R2</x:v>
+        <x:v>Lang / Round2</x:v>
       </x:c>
       <x:c r="B37" s="19" t="n">
         <x:v>61</x:v>
@@ -1115,15 +1176,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F37" s="14" t="n">
-        <x:v>79.33</x:v>
+        <x:v>79.32803278688525</x:v>
       </x:c>
       <x:c r="G37" s="14" t="n">
-        <x:v>84.32</x:v>
+        <x:v>84.32409836065574</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="8" t="str">
-        <x:v>Math · R1</x:v>
+        <x:v>Math / Round1</x:v>
       </x:c>
       <x:c r="B38" s="19" t="n">
         <x:v>106</x:v>
@@ -1138,15 +1199,15 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="F38" s="14" t="n">
-        <x:v>81.2</x:v>
+        <x:v>81.19683673469386</x:v>
       </x:c>
       <x:c r="G38" s="14" t="n">
-        <x:v>84.25</x:v>
+        <x:v>84.2484693877551</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="8" t="str">
-        <x:v>Math · R2</x:v>
+        <x:v>Math / Round2</x:v>
       </x:c>
       <x:c r="B39" s="19" t="n">
         <x:v>106</x:v>
@@ -1161,15 +1222,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F39" s="14" t="n">
-        <x:v>81.42</x:v>
+        <x:v>81.42292452830186</x:v>
       </x:c>
       <x:c r="G39" s="14" t="n">
-        <x:v>84.37</x:v>
+        <x:v>84.36669811320755</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="8" t="str">
-        <x:v>Mockito · R1</x:v>
+        <x:v>Mockito / Round1</x:v>
       </x:c>
       <x:c r="B40" s="19" t="n">
         <x:v>38</x:v>
@@ -1184,15 +1245,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F40" s="14" t="n">
-        <x:v>36.18</x:v>
+        <x:v>36.180285714285716</x:v>
       </x:c>
       <x:c r="G40" s="14" t="n">
-        <x:v>52.54</x:v>
+        <x:v>52.54394736842105</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="8" t="str">
-        <x:v>Mockito · R2</x:v>
+        <x:v>Mockito / Round2</x:v>
       </x:c>
       <x:c r="B41" s="19" t="n">
         <x:v>38</x:v>
@@ -1207,15 +1268,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F41" s="14" t="n">
-        <x:v>36.18</x:v>
+        <x:v>36.180285714285716</x:v>
       </x:c>
       <x:c r="G41" s="14" t="n">
-        <x:v>52.54</x:v>
+        <x:v>52.54394736842105</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="8" t="str">
-        <x:v>Time · R1</x:v>
+        <x:v>Time / Round1</x:v>
       </x:c>
       <x:c r="B42" s="19" t="n">
         <x:v>26</x:v>
@@ -1230,15 +1291,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F42" s="14" t="n">
-        <x:v>79.59</x:v>
+        <x:v>79.58961538461539</x:v>
       </x:c>
       <x:c r="G42" s="14" t="n">
-        <x:v>86.87</x:v>
+        <x:v>86.8726923076923</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="8" t="str">
-        <x:v>Time · R2</x:v>
+        <x:v>Time / Round2</x:v>
       </x:c>
       <x:c r="B43" s="19" t="n">
         <x:v>26</x:v>
@@ -1253,13 +1314,230 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F43" s="14" t="n">
-        <x:v>79.59</x:v>
+        <x:v>79.58961538461539</x:v>
       </x:c>
       <x:c r="G43" s="14" t="n">
-        <x:v>86.87</x:v>
+        <x:v>86.8726923076923</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="B48" s="28" t="str">
+        <x:v>Coverage — recorded values and all saved results</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="B49" t="str">
+        <x:v>Recorded only excludes blanks. All results counts blanks as 0%. See Coverage for every project.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="42" customHeight="1">
+      <x:c r="B51" s="31" t="str">
+        <x:v>Project</x:v>
+      </x:c>
+      <x:c r="C51" s="31" t="str">
+        <x:v>Round</x:v>
+      </x:c>
+      <x:c r="D51" s="31" t="str">
+        <x:v>Metric</x:v>
+      </x:c>
+      <x:c r="E51" s="31" t="str">
+        <x:v>Results</x:v>
+      </x:c>
+      <x:c r="F51" s="31" t="str">
+        <x:v>Recorded values</x:v>
+      </x:c>
+      <x:c r="G51" s="31" t="str">
+        <x:v>Recorded only</x:v>
+      </x:c>
+      <x:c r="H51" s="31" t="str">
+        <x:v>All results (missing = 0%)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="23" customHeight="1">
+      <x:c r="B52" s="22" t="str">
+        <x:f>'Coverage'!B7</x:f>
+        <x:v>All projects</x:v>
+      </x:c>
+      <x:c r="C52" s="22" t="str">
+        <x:f>'Coverage'!C7</x:f>
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D52" s="22" t="str">
+        <x:f>'Coverage'!D7</x:f>
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E52" s="26" t="n">
+        <x:f>'Coverage'!E7</x:f>
+        <x:v>1702</x:v>
+      </x:c>
+      <x:c r="F52" s="26" t="n">
+        <x:f>'Coverage'!F7</x:f>
+        <x:v>1634</x:v>
+      </x:c>
+      <x:c r="G52" s="27" t="n">
+        <x:f>'Coverage'!G7</x:f>
+        <x:v>0.6154589963280295</x:v>
+      </x:c>
+      <x:c r="H52" s="27" t="n">
+        <x:f>'Coverage'!H7</x:f>
+        <x:v>0.5908695652173914</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="23" customHeight="1">
+      <x:c r="B53" s="22" t="str">
+        <x:f>'Coverage'!B8</x:f>
+        <x:v>All projects</x:v>
+      </x:c>
+      <x:c r="C53" s="22" t="str">
+        <x:f>'Coverage'!C8</x:f>
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D53" s="22" t="str">
+        <x:f>'Coverage'!D8</x:f>
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E53" s="26" t="n">
+        <x:f>'Coverage'!E8</x:f>
+        <x:v>1702</x:v>
+      </x:c>
+      <x:c r="F53" s="26" t="n">
+        <x:f>'Coverage'!F8</x:f>
+        <x:v>1626</x:v>
+      </x:c>
+      <x:c r="G53" s="27" t="n">
+        <x:f>'Coverage'!G8</x:f>
+        <x:v>0.5391292742927433</x:v>
+      </x:c>
+      <x:c r="H53" s="27" t="n">
+        <x:f>'Coverage'!H8</x:f>
+        <x:v>0.5150553466509992</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="23" customHeight="1">
+      <x:c r="B54" s="22" t="str">
+        <x:f>'Coverage'!B9</x:f>
+        <x:v>All projects</x:v>
+      </x:c>
+      <x:c r="C54" s="22" t="str">
+        <x:f>'Coverage'!C9</x:f>
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D54" s="22" t="str">
+        <x:f>'Coverage'!D9</x:f>
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E54" s="26" t="n">
+        <x:f>'Coverage'!E9</x:f>
+        <x:v>851</x:v>
+      </x:c>
+      <x:c r="F54" s="26" t="n">
+        <x:f>'Coverage'!F9</x:f>
+        <x:v>813</x:v>
+      </x:c>
+      <x:c r="G54" s="27" t="n">
+        <x:f>'Coverage'!G9</x:f>
+        <x:v>0.6142649446494468</x:v>
+      </x:c>
+      <x:c r="H54" s="27" t="n">
+        <x:f>'Coverage'!H9</x:f>
+        <x:v>0.5868359576968276</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="23" customHeight="1">
+      <x:c r="B55" s="22" t="str">
+        <x:f>'Coverage'!B10</x:f>
+        <x:v>All projects</x:v>
+      </x:c>
+      <x:c r="C55" s="22" t="str">
+        <x:f>'Coverage'!C10</x:f>
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D55" s="22" t="str">
+        <x:f>'Coverage'!D10</x:f>
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E55" s="26" t="n">
+        <x:f>'Coverage'!E10</x:f>
+        <x:v>851</x:v>
+      </x:c>
+      <x:c r="F55" s="26" t="n">
+        <x:f>'Coverage'!F10</x:f>
+        <x:v>809</x:v>
+      </x:c>
+      <x:c r="G55" s="27" t="n">
+        <x:f>'Coverage'!G10</x:f>
+        <x:v>0.5376321384425218</x:v>
+      </x:c>
+      <x:c r="H55" s="27" t="n">
+        <x:f>'Coverage'!H10</x:f>
+        <x:v>0.5110980023501763</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="23" customHeight="1">
+      <x:c r="B56" s="22" t="str">
+        <x:f>'Coverage'!B11</x:f>
+        <x:v>All projects</x:v>
+      </x:c>
+      <x:c r="C56" s="22" t="str">
+        <x:f>'Coverage'!C11</x:f>
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D56" s="22" t="str">
+        <x:f>'Coverage'!D11</x:f>
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E56" s="26" t="n">
+        <x:f>'Coverage'!E11</x:f>
+        <x:v>851</x:v>
+      </x:c>
+      <x:c r="F56" s="26" t="n">
+        <x:f>'Coverage'!F11</x:f>
+        <x:v>821</x:v>
+      </x:c>
+      <x:c r="G56" s="27" t="n">
+        <x:f>'Coverage'!G11</x:f>
+        <x:v>0.6166414129110843</x:v>
+      </x:c>
+      <x:c r="H56" s="27" t="n">
+        <x:f>'Coverage'!H11</x:f>
+        <x:v>0.5949031727379556</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="23" customHeight="1">
+      <x:c r="B57" s="22" t="str">
+        <x:f>'Coverage'!B12</x:f>
+        <x:v>All projects</x:v>
+      </x:c>
+      <x:c r="C57" s="22" t="str">
+        <x:f>'Coverage'!C12</x:f>
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D57" s="22" t="str">
+        <x:f>'Coverage'!D12</x:f>
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E57" s="26" t="n">
+        <x:f>'Coverage'!E12</x:f>
+        <x:v>851</x:v>
+      </x:c>
+      <x:c r="F57" s="26" t="n">
+        <x:f>'Coverage'!F12</x:f>
+        <x:v>817</x:v>
+      </x:c>
+      <x:c r="G57" s="27" t="n">
+        <x:f>'Coverage'!G12</x:f>
+        <x:v>0.5406117503059977</x:v>
+      </x:c>
+      <x:c r="H57" s="27" t="n">
+        <x:f>'Coverage'!H12</x:f>
+        <x:v>0.5190126909518216</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="B48:H48"/>
+    <x:mergeCell ref="B49:H49"/>
+  </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -65031,7 +65309,2983 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R818d3bde7a9c4d34"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R135f70a011dd4db0"/>
   </x:tableParts>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="2" max="2" width="29" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="23" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="23" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="2">
+      <x:c r="B2" s="21" t="str">
+        <x:v>Coverage by project and round</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="B3" t="str">
+        <x:v>Recorded: numeric values only. All results: missing coverage counts as 0%.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="B4" t="str">
+        <x:v>Each saved result is one case. A target in two rounds counts twice. Raw blanks remain blank.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="42" customHeight="1">
+      <x:c r="B6" s="31" t="str">
+        <x:v>Project</x:v>
+      </x:c>
+      <x:c r="C6" s="31" t="str">
+        <x:v>Round</x:v>
+      </x:c>
+      <x:c r="D6" s="31" t="str">
+        <x:v>Metric</x:v>
+      </x:c>
+      <x:c r="E6" s="31" t="str">
+        <x:v>Results</x:v>
+      </x:c>
+      <x:c r="F6" s="31" t="str">
+        <x:v>Recorded values</x:v>
+      </x:c>
+      <x:c r="G6" s="31" t="str">
+        <x:v>Recorded only</x:v>
+      </x:c>
+      <x:c r="H6" s="31" t="str">
+        <x:v>All results (missing = 0%)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="23" customHeight="1">
+      <x:c r="B7" s="22" t="str">
+        <x:v>All projects</x:v>
+      </x:c>
+      <x:c r="C7" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D7" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E7" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$2:$D$1703)</x:f>
+        <x:v>1702</x:v>
+      </x:c>
+      <x:c r="F7" s="26" t="n">
+        <x:f>COUNT('Data'!$H$2:$H$1703)</x:f>
+        <x:v>1634</x:v>
+      </x:c>
+      <x:c r="G7" s="27" t="n">
+        <x:f>IF(F7=0,"—",SUM('Data'!$H$2:$H$1703)/F7/100)</x:f>
+        <x:v>0.6154589963280295</x:v>
+      </x:c>
+      <x:c r="H7" s="27" t="n">
+        <x:f>IF(E7=0,"—",SUM('Data'!$H$2:$H$1703)/E7/100)</x:f>
+        <x:v>0.5908695652173914</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="23" customHeight="1">
+      <x:c r="B8" s="22" t="str">
+        <x:v>All projects</x:v>
+      </x:c>
+      <x:c r="C8" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D8" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E8" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$2:$D$1703)</x:f>
+        <x:v>1702</x:v>
+      </x:c>
+      <x:c r="F8" s="26" t="n">
+        <x:f>COUNT('Data'!$K$2:$K$1703)</x:f>
+        <x:v>1626</x:v>
+      </x:c>
+      <x:c r="G8" s="27" t="n">
+        <x:f>IF(F8=0,"—",SUM('Data'!$K$2:$K$1703)/F8/100)</x:f>
+        <x:v>0.5391292742927433</x:v>
+      </x:c>
+      <x:c r="H8" s="27" t="n">
+        <x:f>IF(E8=0,"—",SUM('Data'!$K$2:$K$1703)/E8/100)</x:f>
+        <x:v>0.5150553466509992</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="23" customHeight="1">
+      <x:c r="B9" s="22" t="str">
+        <x:v>All projects</x:v>
+      </x:c>
+      <x:c r="C9" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D9" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E9" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$2:$D$852)</x:f>
+        <x:v>851</x:v>
+      </x:c>
+      <x:c r="F9" s="26" t="n">
+        <x:f>COUNT('Data'!$H$2:$H$852)</x:f>
+        <x:v>813</x:v>
+      </x:c>
+      <x:c r="G9" s="27" t="n">
+        <x:f>IF(F9=0,"—",SUM('Data'!$H$2:$H$852)/F9/100)</x:f>
+        <x:v>0.6142649446494468</x:v>
+      </x:c>
+      <x:c r="H9" s="27" t="n">
+        <x:f>IF(E9=0,"—",SUM('Data'!$H$2:$H$852)/E9/100)</x:f>
+        <x:v>0.5868359576968276</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="23" customHeight="1">
+      <x:c r="B10" s="22" t="str">
+        <x:v>All projects</x:v>
+      </x:c>
+      <x:c r="C10" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D10" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E10" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$2:$D$852)</x:f>
+        <x:v>851</x:v>
+      </x:c>
+      <x:c r="F10" s="26" t="n">
+        <x:f>COUNT('Data'!$K$2:$K$852)</x:f>
+        <x:v>809</x:v>
+      </x:c>
+      <x:c r="G10" s="27" t="n">
+        <x:f>IF(F10=0,"—",SUM('Data'!$K$2:$K$852)/F10/100)</x:f>
+        <x:v>0.5376321384425218</x:v>
+      </x:c>
+      <x:c r="H10" s="27" t="n">
+        <x:f>IF(E10=0,"—",SUM('Data'!$K$2:$K$852)/E10/100)</x:f>
+        <x:v>0.5110980023501763</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="23" customHeight="1">
+      <x:c r="B11" s="22" t="str">
+        <x:v>All projects</x:v>
+      </x:c>
+      <x:c r="C11" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D11" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E11" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$853:$D$1703)</x:f>
+        <x:v>851</x:v>
+      </x:c>
+      <x:c r="F11" s="26" t="n">
+        <x:f>COUNT('Data'!$H$853:$H$1703)</x:f>
+        <x:v>821</x:v>
+      </x:c>
+      <x:c r="G11" s="27" t="n">
+        <x:f>IF(F11=0,"—",SUM('Data'!$H$853:$H$1703)/F11/100)</x:f>
+        <x:v>0.6166414129110843</x:v>
+      </x:c>
+      <x:c r="H11" s="27" t="n">
+        <x:f>IF(E11=0,"—",SUM('Data'!$H$853:$H$1703)/E11/100)</x:f>
+        <x:v>0.5949031727379556</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="23" customHeight="1">
+      <x:c r="B12" s="22" t="str">
+        <x:v>All projects</x:v>
+      </x:c>
+      <x:c r="C12" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D12" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E12" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$853:$D$1703)</x:f>
+        <x:v>851</x:v>
+      </x:c>
+      <x:c r="F12" s="26" t="n">
+        <x:f>COUNT('Data'!$K$853:$K$1703)</x:f>
+        <x:v>817</x:v>
+      </x:c>
+      <x:c r="G12" s="27" t="n">
+        <x:f>IF(F12=0,"—",SUM('Data'!$K$853:$K$1703)/F12/100)</x:f>
+        <x:v>0.5406117503059977</x:v>
+      </x:c>
+      <x:c r="H12" s="27" t="n">
+        <x:f>IF(E12=0,"—",SUM('Data'!$K$853:$K$1703)/E12/100)</x:f>
+        <x:v>0.5190126909518216</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="23" customHeight="1">
+      <x:c r="B13" s="22" t="str">
+        <x:v>Chart</x:v>
+      </x:c>
+      <x:c r="C13" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D13" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E13" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$2:$D$27,'Data'!$D$853:$D$878)</x:f>
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="F13" s="26" t="n">
+        <x:f>COUNT('Data'!$H$2:$H$27,'Data'!$H$853:$H$878)</x:f>
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="G13" s="27" t="n">
+        <x:f>IF(F13=0,"—",SUM('Data'!$H$2:$H$27,'Data'!$H$853:$H$878)/F13/100)</x:f>
+        <x:v>0.779023076923077</x:v>
+      </x:c>
+      <x:c r="H13" s="27" t="n">
+        <x:f>IF(E13=0,"—",SUM('Data'!$H$2:$H$27,'Data'!$H$853:$H$878)/E13/100)</x:f>
+        <x:v>0.779023076923077</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="23" customHeight="1">
+      <x:c r="B14" s="22" t="str">
+        <x:v>Chart</x:v>
+      </x:c>
+      <x:c r="C14" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D14" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E14" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$2:$D$27,'Data'!$D$853:$D$878)</x:f>
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="F14" s="26" t="n">
+        <x:f>COUNT('Data'!$K$2:$K$27,'Data'!$K$853:$K$878)</x:f>
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="G14" s="27" t="n">
+        <x:f>IF(F14=0,"—",SUM('Data'!$K$2:$K$27,'Data'!$K$853:$K$878)/F14/100)</x:f>
+        <x:v>0.705304</x:v>
+      </x:c>
+      <x:c r="H14" s="27" t="n">
+        <x:f>IF(E14=0,"—",SUM('Data'!$K$2:$K$27,'Data'!$K$853:$K$878)/E14/100)</x:f>
+        <x:v>0.6781769230769231</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="23" customHeight="1">
+      <x:c r="B15" s="22" t="str">
+        <x:v>Chart</x:v>
+      </x:c>
+      <x:c r="C15" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D15" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E15" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$2:$D$27)</x:f>
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="F15" s="26" t="n">
+        <x:f>COUNT('Data'!$H$2:$H$27)</x:f>
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="G15" s="27" t="n">
+        <x:f>IF(F15=0,"—",SUM('Data'!$H$2:$H$27)/F15/100)</x:f>
+        <x:v>0.779023076923077</x:v>
+      </x:c>
+      <x:c r="H15" s="27" t="n">
+        <x:f>IF(E15=0,"—",SUM('Data'!$H$2:$H$27)/E15/100)</x:f>
+        <x:v>0.779023076923077</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="23" customHeight="1">
+      <x:c r="B16" s="22" t="str">
+        <x:v>Chart</x:v>
+      </x:c>
+      <x:c r="C16" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D16" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E16" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$2:$D$27)</x:f>
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="F16" s="26" t="n">
+        <x:f>COUNT('Data'!$K$2:$K$27)</x:f>
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="G16" s="27" t="n">
+        <x:f>IF(F16=0,"—",SUM('Data'!$K$2:$K$27)/F16/100)</x:f>
+        <x:v>0.705304</x:v>
+      </x:c>
+      <x:c r="H16" s="27" t="n">
+        <x:f>IF(E16=0,"—",SUM('Data'!$K$2:$K$27)/E16/100)</x:f>
+        <x:v>0.6781769230769231</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="23" customHeight="1">
+      <x:c r="B17" s="22" t="str">
+        <x:v>Chart</x:v>
+      </x:c>
+      <x:c r="C17" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D17" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E17" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$853:$D$878)</x:f>
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="F17" s="26" t="n">
+        <x:f>COUNT('Data'!$H$853:$H$878)</x:f>
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="G17" s="27" t="n">
+        <x:f>IF(F17=0,"—",SUM('Data'!$H$853:$H$878)/F17/100)</x:f>
+        <x:v>0.779023076923077</x:v>
+      </x:c>
+      <x:c r="H17" s="27" t="n">
+        <x:f>IF(E17=0,"—",SUM('Data'!$H$853:$H$878)/E17/100)</x:f>
+        <x:v>0.779023076923077</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="23" customHeight="1">
+      <x:c r="B18" s="22" t="str">
+        <x:v>Chart</x:v>
+      </x:c>
+      <x:c r="C18" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D18" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E18" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$853:$D$878)</x:f>
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="F18" s="26" t="n">
+        <x:f>COUNT('Data'!$K$853:$K$878)</x:f>
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="G18" s="27" t="n">
+        <x:f>IF(F18=0,"—",SUM('Data'!$K$853:$K$878)/F18/100)</x:f>
+        <x:v>0.705304</x:v>
+      </x:c>
+      <x:c r="H18" s="27" t="n">
+        <x:f>IF(E18=0,"—",SUM('Data'!$K$853:$K$878)/E18/100)</x:f>
+        <x:v>0.6781769230769231</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="23" customHeight="1">
+      <x:c r="B19" s="22" t="str">
+        <x:v>Cli</x:v>
+      </x:c>
+      <x:c r="C19" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D19" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E19" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$28:$D$66,'Data'!$D$879:$D$917)</x:f>
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="F19" s="26" t="n">
+        <x:f>COUNT('Data'!$H$28:$H$66,'Data'!$H$879:$H$917)</x:f>
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="G19" s="27" t="n">
+        <x:f>IF(F19=0,"—",SUM('Data'!$H$28:$H$66,'Data'!$H$879:$H$917)/F19/100)</x:f>
+        <x:v>0.1339897435897436</x:v>
+      </x:c>
+      <x:c r="H19" s="27" t="n">
+        <x:f>IF(E19=0,"—",SUM('Data'!$H$28:$H$66,'Data'!$H$879:$H$917)/E19/100)</x:f>
+        <x:v>0.1339897435897436</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="23" customHeight="1">
+      <x:c r="B20" s="22" t="str">
+        <x:v>Cli</x:v>
+      </x:c>
+      <x:c r="C20" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D20" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E20" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$28:$D$66,'Data'!$D$879:$D$917)</x:f>
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="F20" s="26" t="n">
+        <x:f>COUNT('Data'!$K$28:$K$66,'Data'!$K$879:$K$917)</x:f>
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="G20" s="27" t="n">
+        <x:f>IF(F20=0,"—",SUM('Data'!$K$28:$K$66,'Data'!$K$879:$K$917)/F20/100)</x:f>
+        <x:v>0.12038205128205128</x:v>
+      </x:c>
+      <x:c r="H20" s="27" t="n">
+        <x:f>IF(E20=0,"—",SUM('Data'!$K$28:$K$66,'Data'!$K$879:$K$917)/E20/100)</x:f>
+        <x:v>0.12038205128205128</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="23" customHeight="1">
+      <x:c r="B21" s="22" t="str">
+        <x:v>Cli</x:v>
+      </x:c>
+      <x:c r="C21" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D21" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E21" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$28:$D$66)</x:f>
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="F21" s="26" t="n">
+        <x:f>COUNT('Data'!$H$28:$H$66)</x:f>
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="G21" s="27" t="n">
+        <x:f>IF(F21=0,"—",SUM('Data'!$H$28:$H$66)/F21/100)</x:f>
+        <x:v>0.1339897435897436</x:v>
+      </x:c>
+      <x:c r="H21" s="27" t="n">
+        <x:f>IF(E21=0,"—",SUM('Data'!$H$28:$H$66)/E21/100)</x:f>
+        <x:v>0.1339897435897436</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="23" customHeight="1">
+      <x:c r="B22" s="22" t="str">
+        <x:v>Cli</x:v>
+      </x:c>
+      <x:c r="C22" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D22" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E22" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$28:$D$66)</x:f>
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="F22" s="26" t="n">
+        <x:f>COUNT('Data'!$K$28:$K$66)</x:f>
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="G22" s="27" t="n">
+        <x:f>IF(F22=0,"—",SUM('Data'!$K$28:$K$66)/F22/100)</x:f>
+        <x:v>0.12038205128205128</x:v>
+      </x:c>
+      <x:c r="H22" s="27" t="n">
+        <x:f>IF(E22=0,"—",SUM('Data'!$K$28:$K$66)/E22/100)</x:f>
+        <x:v>0.12038205128205128</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="23" customHeight="1">
+      <x:c r="B23" s="22" t="str">
+        <x:v>Cli</x:v>
+      </x:c>
+      <x:c r="C23" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D23" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E23" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$879:$D$917)</x:f>
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="F23" s="26" t="n">
+        <x:f>COUNT('Data'!$H$879:$H$917)</x:f>
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="G23" s="27" t="n">
+        <x:f>IF(F23=0,"—",SUM('Data'!$H$879:$H$917)/F23/100)</x:f>
+        <x:v>0.1339897435897436</x:v>
+      </x:c>
+      <x:c r="H23" s="27" t="n">
+        <x:f>IF(E23=0,"—",SUM('Data'!$H$879:$H$917)/E23/100)</x:f>
+        <x:v>0.1339897435897436</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="23" customHeight="1">
+      <x:c r="B24" s="22" t="str">
+        <x:v>Cli</x:v>
+      </x:c>
+      <x:c r="C24" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D24" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E24" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$879:$D$917)</x:f>
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="F24" s="26" t="n">
+        <x:f>COUNT('Data'!$K$879:$K$917)</x:f>
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="G24" s="27" t="n">
+        <x:f>IF(F24=0,"—",SUM('Data'!$K$879:$K$917)/F24/100)</x:f>
+        <x:v>0.12038205128205128</x:v>
+      </x:c>
+      <x:c r="H24" s="27" t="n">
+        <x:f>IF(E24=0,"—",SUM('Data'!$K$879:$K$917)/E24/100)</x:f>
+        <x:v>0.12038205128205128</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="23" customHeight="1">
+      <x:c r="B25" s="22" t="str">
+        <x:v>Closure</x:v>
+      </x:c>
+      <x:c r="C25" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D25" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E25" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$67:$D$240,'Data'!$D$918:$D$1091)</x:f>
+        <x:v>348</x:v>
+      </x:c>
+      <x:c r="F25" s="26" t="n">
+        <x:f>COUNT('Data'!$H$67:$H$240,'Data'!$H$918:$H$1091)</x:f>
+        <x:v>294</x:v>
+      </x:c>
+      <x:c r="G25" s="27" t="n">
+        <x:f>IF(F25=0,"—",SUM('Data'!$H$67:$H$240,'Data'!$H$918:$H$1091)/F25/100)</x:f>
+        <x:v>0.31966054421768697</x:v>
+      </x:c>
+      <x:c r="H25" s="27" t="n">
+        <x:f>IF(E25=0,"—",SUM('Data'!$H$67:$H$240,'Data'!$H$918:$H$1091)/E25/100)</x:f>
+        <x:v>0.2700580459770114</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="23" customHeight="1">
+      <x:c r="B26" s="22" t="str">
+        <x:v>Closure</x:v>
+      </x:c>
+      <x:c r="C26" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D26" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E26" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$67:$D$240,'Data'!$D$918:$D$1091)</x:f>
+        <x:v>348</x:v>
+      </x:c>
+      <x:c r="F26" s="26" t="n">
+        <x:f>COUNT('Data'!$K$67:$K$240,'Data'!$K$918:$K$1091)</x:f>
+        <x:v>294</x:v>
+      </x:c>
+      <x:c r="G26" s="27" t="n">
+        <x:f>IF(F26=0,"—",SUM('Data'!$K$67:$K$240,'Data'!$K$918:$K$1091)/F26/100)</x:f>
+        <x:v>0.20511972789115643</x:v>
+      </x:c>
+      <x:c r="H26" s="27" t="n">
+        <x:f>IF(E26=0,"—",SUM('Data'!$K$67:$K$240,'Data'!$K$918:$K$1091)/E26/100)</x:f>
+        <x:v>0.1732908045977011</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="23" customHeight="1">
+      <x:c r="B27" s="22" t="str">
+        <x:v>Closure</x:v>
+      </x:c>
+      <x:c r="C27" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D27" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E27" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$67:$D$240)</x:f>
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="F27" s="26" t="n">
+        <x:f>COUNT('Data'!$H$67:$H$240)</x:f>
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="G27" s="27" t="n">
+        <x:f>IF(F27=0,"—",SUM('Data'!$H$67:$H$240)/F27/100)</x:f>
+        <x:v>0.31966054421768697</x:v>
+      </x:c>
+      <x:c r="H27" s="27" t="n">
+        <x:f>IF(E27=0,"—",SUM('Data'!$H$67:$H$240)/E27/100)</x:f>
+        <x:v>0.2700580459770114</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="23" customHeight="1">
+      <x:c r="B28" s="22" t="str">
+        <x:v>Closure</x:v>
+      </x:c>
+      <x:c r="C28" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D28" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E28" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$67:$D$240)</x:f>
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="F28" s="26" t="n">
+        <x:f>COUNT('Data'!$K$67:$K$240)</x:f>
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="G28" s="27" t="n">
+        <x:f>IF(F28=0,"—",SUM('Data'!$K$67:$K$240)/F28/100)</x:f>
+        <x:v>0.20511972789115643</x:v>
+      </x:c>
+      <x:c r="H28" s="27" t="n">
+        <x:f>IF(E28=0,"—",SUM('Data'!$K$67:$K$240)/E28/100)</x:f>
+        <x:v>0.1732908045977011</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="23" customHeight="1">
+      <x:c r="B29" s="22" t="str">
+        <x:v>Closure</x:v>
+      </x:c>
+      <x:c r="C29" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D29" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E29" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$918:$D$1091)</x:f>
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="F29" s="26" t="n">
+        <x:f>COUNT('Data'!$H$918:$H$1091)</x:f>
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="G29" s="27" t="n">
+        <x:f>IF(F29=0,"—",SUM('Data'!$H$918:$H$1091)/F29/100)</x:f>
+        <x:v>0.31966054421768697</x:v>
+      </x:c>
+      <x:c r="H29" s="27" t="n">
+        <x:f>IF(E29=0,"—",SUM('Data'!$H$918:$H$1091)/E29/100)</x:f>
+        <x:v>0.2700580459770114</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="23" customHeight="1">
+      <x:c r="B30" s="22" t="str">
+        <x:v>Closure</x:v>
+      </x:c>
+      <x:c r="C30" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D30" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E30" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$918:$D$1091)</x:f>
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="F30" s="26" t="n">
+        <x:f>COUNT('Data'!$K$918:$K$1091)</x:f>
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="G30" s="27" t="n">
+        <x:f>IF(F30=0,"—",SUM('Data'!$K$918:$K$1091)/F30/100)</x:f>
+        <x:v>0.20511972789115643</x:v>
+      </x:c>
+      <x:c r="H30" s="27" t="n">
+        <x:f>IF(E30=0,"—",SUM('Data'!$K$918:$K$1091)/E30/100)</x:f>
+        <x:v>0.1732908045977011</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="23" customHeight="1">
+      <x:c r="B31" s="22" t="str">
+        <x:v>Codec</x:v>
+      </x:c>
+      <x:c r="C31" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D31" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E31" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$241:$D$258,'Data'!$D$1092:$D$1109)</x:f>
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="F31" s="26" t="n">
+        <x:f>COUNT('Data'!$H$241:$H$258,'Data'!$H$1092:$H$1109)</x:f>
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="G31" s="27" t="n">
+        <x:f>IF(F31=0,"—",SUM('Data'!$H$241:$H$258,'Data'!$H$1092:$H$1109)/F31/100)</x:f>
+        <x:v>0.8786888888888889</x:v>
+      </x:c>
+      <x:c r="H31" s="27" t="n">
+        <x:f>IF(E31=0,"—",SUM('Data'!$H$241:$H$258,'Data'!$H$1092:$H$1109)/E31/100)</x:f>
+        <x:v>0.8786888888888889</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="23" customHeight="1">
+      <x:c r="B32" s="22" t="str">
+        <x:v>Codec</x:v>
+      </x:c>
+      <x:c r="C32" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D32" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E32" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$241:$D$258,'Data'!$D$1092:$D$1109)</x:f>
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="F32" s="26" t="n">
+        <x:f>COUNT('Data'!$K$241:$K$258,'Data'!$K$1092:$K$1109)</x:f>
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="G32" s="27" t="n">
+        <x:f>IF(F32=0,"—",SUM('Data'!$K$241:$K$258,'Data'!$K$1092:$K$1109)/F32/100)</x:f>
+        <x:v>0.8367444444444445</x:v>
+      </x:c>
+      <x:c r="H32" s="27" t="n">
+        <x:f>IF(E32=0,"—",SUM('Data'!$K$241:$K$258,'Data'!$K$1092:$K$1109)/E32/100)</x:f>
+        <x:v>0.8367444444444445</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="23" customHeight="1">
+      <x:c r="B33" s="22" t="str">
+        <x:v>Codec</x:v>
+      </x:c>
+      <x:c r="C33" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D33" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E33" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$241:$D$258)</x:f>
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F33" s="26" t="n">
+        <x:f>COUNT('Data'!$H$241:$H$258)</x:f>
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="G33" s="27" t="n">
+        <x:f>IF(F33=0,"—",SUM('Data'!$H$241:$H$258)/F33/100)</x:f>
+        <x:v>0.8786888888888889</x:v>
+      </x:c>
+      <x:c r="H33" s="27" t="n">
+        <x:f>IF(E33=0,"—",SUM('Data'!$H$241:$H$258)/E33/100)</x:f>
+        <x:v>0.8786888888888889</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="23" customHeight="1">
+      <x:c r="B34" s="22" t="str">
+        <x:v>Codec</x:v>
+      </x:c>
+      <x:c r="C34" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D34" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E34" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$241:$D$258)</x:f>
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F34" s="26" t="n">
+        <x:f>COUNT('Data'!$K$241:$K$258)</x:f>
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="G34" s="27" t="n">
+        <x:f>IF(F34=0,"—",SUM('Data'!$K$241:$K$258)/F34/100)</x:f>
+        <x:v>0.8367444444444445</x:v>
+      </x:c>
+      <x:c r="H34" s="27" t="n">
+        <x:f>IF(E34=0,"—",SUM('Data'!$K$241:$K$258)/E34/100)</x:f>
+        <x:v>0.8367444444444445</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="23" customHeight="1">
+      <x:c r="B35" s="22" t="str">
+        <x:v>Codec</x:v>
+      </x:c>
+      <x:c r="C35" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D35" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E35" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$1092:$D$1109)</x:f>
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F35" s="26" t="n">
+        <x:f>COUNT('Data'!$H$1092:$H$1109)</x:f>
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="G35" s="27" t="n">
+        <x:f>IF(F35=0,"—",SUM('Data'!$H$1092:$H$1109)/F35/100)</x:f>
+        <x:v>0.8786888888888889</x:v>
+      </x:c>
+      <x:c r="H35" s="27" t="n">
+        <x:f>IF(E35=0,"—",SUM('Data'!$H$1092:$H$1109)/E35/100)</x:f>
+        <x:v>0.8786888888888889</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="23" customHeight="1">
+      <x:c r="B36" s="22" t="str">
+        <x:v>Codec</x:v>
+      </x:c>
+      <x:c r="C36" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D36" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E36" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$1092:$D$1109)</x:f>
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F36" s="26" t="n">
+        <x:f>COUNT('Data'!$K$1092:$K$1109)</x:f>
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="G36" s="27" t="n">
+        <x:f>IF(F36=0,"—",SUM('Data'!$K$1092:$K$1109)/F36/100)</x:f>
+        <x:v>0.8367444444444445</x:v>
+      </x:c>
+      <x:c r="H36" s="27" t="n">
+        <x:f>IF(E36=0,"—",SUM('Data'!$K$1092:$K$1109)/E36/100)</x:f>
+        <x:v>0.8367444444444445</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="23" customHeight="1">
+      <x:c r="B37" s="22" t="str">
+        <x:v>Collections</x:v>
+      </x:c>
+      <x:c r="C37" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D37" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E37" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$259:$D$286,'Data'!$D$1110:$D$1137)</x:f>
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="F37" s="26" t="n">
+        <x:f>COUNT('Data'!$H$259:$H$286,'Data'!$H$1110:$H$1137)</x:f>
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="G37" s="27" t="n">
+        <x:f>IF(F37=0,"—",SUM('Data'!$H$259:$H$286,'Data'!$H$1110:$H$1137)/F37/100)</x:f>
+        <x:v>0.8044571428571429</x:v>
+      </x:c>
+      <x:c r="H37" s="27" t="n">
+        <x:f>IF(E37=0,"—",SUM('Data'!$H$259:$H$286,'Data'!$H$1110:$H$1137)/E37/100)</x:f>
+        <x:v>0.8044571428571429</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="23" customHeight="1">
+      <x:c r="B38" s="22" t="str">
+        <x:v>Collections</x:v>
+      </x:c>
+      <x:c r="C38" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D38" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E38" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$259:$D$286,'Data'!$D$1110:$D$1137)</x:f>
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="F38" s="26" t="n">
+        <x:f>COUNT('Data'!$K$259:$K$286,'Data'!$K$1110:$K$1137)</x:f>
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="G38" s="27" t="n">
+        <x:f>IF(F38=0,"—",SUM('Data'!$K$259:$K$286,'Data'!$K$1110:$K$1137)/F38/100)</x:f>
+        <x:v>0.7924071428571429</x:v>
+      </x:c>
+      <x:c r="H38" s="27" t="n">
+        <x:f>IF(E38=0,"—",SUM('Data'!$K$259:$K$286,'Data'!$K$1110:$K$1137)/E38/100)</x:f>
+        <x:v>0.7924071428571429</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="23" customHeight="1">
+      <x:c r="B39" s="22" t="str">
+        <x:v>Collections</x:v>
+      </x:c>
+      <x:c r="C39" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D39" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E39" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$259:$D$286)</x:f>
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="F39" s="26" t="n">
+        <x:f>COUNT('Data'!$H$259:$H$286)</x:f>
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="G39" s="27" t="n">
+        <x:f>IF(F39=0,"—",SUM('Data'!$H$259:$H$286)/F39/100)</x:f>
+        <x:v>0.8044571428571429</x:v>
+      </x:c>
+      <x:c r="H39" s="27" t="n">
+        <x:f>IF(E39=0,"—",SUM('Data'!$H$259:$H$286)/E39/100)</x:f>
+        <x:v>0.8044571428571429</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="23" customHeight="1">
+      <x:c r="B40" s="22" t="str">
+        <x:v>Collections</x:v>
+      </x:c>
+      <x:c r="C40" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D40" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E40" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$259:$D$286)</x:f>
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="F40" s="26" t="n">
+        <x:f>COUNT('Data'!$K$259:$K$286)</x:f>
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="G40" s="27" t="n">
+        <x:f>IF(F40=0,"—",SUM('Data'!$K$259:$K$286)/F40/100)</x:f>
+        <x:v>0.7924071428571429</x:v>
+      </x:c>
+      <x:c r="H40" s="27" t="n">
+        <x:f>IF(E40=0,"—",SUM('Data'!$K$259:$K$286)/E40/100)</x:f>
+        <x:v>0.7924071428571429</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="23" customHeight="1">
+      <x:c r="B41" s="22" t="str">
+        <x:v>Collections</x:v>
+      </x:c>
+      <x:c r="C41" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D41" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E41" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$1110:$D$1137)</x:f>
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="F41" s="26" t="n">
+        <x:f>COUNT('Data'!$H$1110:$H$1137)</x:f>
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="G41" s="27" t="n">
+        <x:f>IF(F41=0,"—",SUM('Data'!$H$1110:$H$1137)/F41/100)</x:f>
+        <x:v>0.8044571428571429</x:v>
+      </x:c>
+      <x:c r="H41" s="27" t="n">
+        <x:f>IF(E41=0,"—",SUM('Data'!$H$1110:$H$1137)/E41/100)</x:f>
+        <x:v>0.8044571428571429</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="23" customHeight="1">
+      <x:c r="B42" s="22" t="str">
+        <x:v>Collections</x:v>
+      </x:c>
+      <x:c r="C42" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D42" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E42" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$1110:$D$1137)</x:f>
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="F42" s="26" t="n">
+        <x:f>COUNT('Data'!$K$1110:$K$1137)</x:f>
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="G42" s="27" t="n">
+        <x:f>IF(F42=0,"—",SUM('Data'!$K$1110:$K$1137)/F42/100)</x:f>
+        <x:v>0.7924071428571429</x:v>
+      </x:c>
+      <x:c r="H42" s="27" t="n">
+        <x:f>IF(E42=0,"—",SUM('Data'!$K$1110:$K$1137)/E42/100)</x:f>
+        <x:v>0.7924071428571429</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="23" customHeight="1">
+      <x:c r="B43" s="22" t="str">
+        <x:v>Compress</x:v>
+      </x:c>
+      <x:c r="C43" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D43" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E43" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$287:$D$333,'Data'!$D$1138:$D$1184)</x:f>
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="F43" s="26" t="n">
+        <x:f>COUNT('Data'!$H$287:$H$333,'Data'!$H$1138:$H$1184)</x:f>
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="G43" s="27" t="n">
+        <x:f>IF(F43=0,"—",SUM('Data'!$H$287:$H$333,'Data'!$H$1138:$H$1184)/F43/100)</x:f>
+        <x:v>0.6618999999999998</x:v>
+      </x:c>
+      <x:c r="H43" s="27" t="n">
+        <x:f>IF(E43=0,"—",SUM('Data'!$H$287:$H$333,'Data'!$H$1138:$H$1184)/E43/100)</x:f>
+        <x:v>0.6618999999999998</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="23" customHeight="1">
+      <x:c r="B44" s="22" t="str">
+        <x:v>Compress</x:v>
+      </x:c>
+      <x:c r="C44" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D44" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E44" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$287:$D$333,'Data'!$D$1138:$D$1184)</x:f>
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="F44" s="26" t="n">
+        <x:f>COUNT('Data'!$K$287:$K$333,'Data'!$K$1138:$K$1184)</x:f>
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="G44" s="27" t="n">
+        <x:f>IF(F44=0,"—",SUM('Data'!$K$287:$K$333,'Data'!$K$1138:$K$1184)/F44/100)</x:f>
+        <x:v>0.6205872340425531</x:v>
+      </x:c>
+      <x:c r="H44" s="27" t="n">
+        <x:f>IF(E44=0,"—",SUM('Data'!$K$287:$K$333,'Data'!$K$1138:$K$1184)/E44/100)</x:f>
+        <x:v>0.6205872340425531</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="23" customHeight="1">
+      <x:c r="B45" s="22" t="str">
+        <x:v>Compress</x:v>
+      </x:c>
+      <x:c r="C45" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D45" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E45" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$287:$D$333)</x:f>
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="F45" s="26" t="n">
+        <x:f>COUNT('Data'!$H$287:$H$333)</x:f>
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="G45" s="27" t="n">
+        <x:f>IF(F45=0,"—",SUM('Data'!$H$287:$H$333)/F45/100)</x:f>
+        <x:v>0.6618999999999998</x:v>
+      </x:c>
+      <x:c r="H45" s="27" t="n">
+        <x:f>IF(E45=0,"—",SUM('Data'!$H$287:$H$333)/E45/100)</x:f>
+        <x:v>0.6618999999999998</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="23" customHeight="1">
+      <x:c r="B46" s="22" t="str">
+        <x:v>Compress</x:v>
+      </x:c>
+      <x:c r="C46" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D46" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E46" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$287:$D$333)</x:f>
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="F46" s="26" t="n">
+        <x:f>COUNT('Data'!$K$287:$K$333)</x:f>
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="G46" s="27" t="n">
+        <x:f>IF(F46=0,"—",SUM('Data'!$K$287:$K$333)/F46/100)</x:f>
+        <x:v>0.6205872340425531</x:v>
+      </x:c>
+      <x:c r="H46" s="27" t="n">
+        <x:f>IF(E46=0,"—",SUM('Data'!$K$287:$K$333)/E46/100)</x:f>
+        <x:v>0.6205872340425531</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="23" customHeight="1">
+      <x:c r="B47" s="22" t="str">
+        <x:v>Compress</x:v>
+      </x:c>
+      <x:c r="C47" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D47" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E47" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$1138:$D$1184)</x:f>
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="F47" s="26" t="n">
+        <x:f>COUNT('Data'!$H$1138:$H$1184)</x:f>
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="G47" s="27" t="n">
+        <x:f>IF(F47=0,"—",SUM('Data'!$H$1138:$H$1184)/F47/100)</x:f>
+        <x:v>0.6618999999999998</x:v>
+      </x:c>
+      <x:c r="H47" s="27" t="n">
+        <x:f>IF(E47=0,"—",SUM('Data'!$H$1138:$H$1184)/E47/100)</x:f>
+        <x:v>0.6618999999999998</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="23" customHeight="1">
+      <x:c r="B48" s="22" t="str">
+        <x:v>Compress</x:v>
+      </x:c>
+      <x:c r="C48" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D48" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E48" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$1138:$D$1184)</x:f>
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="F48" s="26" t="n">
+        <x:f>COUNT('Data'!$K$1138:$K$1184)</x:f>
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="G48" s="27" t="n">
+        <x:f>IF(F48=0,"—",SUM('Data'!$K$1138:$K$1184)/F48/100)</x:f>
+        <x:v>0.6205872340425531</x:v>
+      </x:c>
+      <x:c r="H48" s="27" t="n">
+        <x:f>IF(E48=0,"—",SUM('Data'!$K$1138:$K$1184)/E48/100)</x:f>
+        <x:v>0.6205872340425531</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="23" customHeight="1">
+      <x:c r="B49" s="22" t="str">
+        <x:v>Csv</x:v>
+      </x:c>
+      <x:c r="C49" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D49" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E49" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$334:$D$349,'Data'!$D$1185:$D$1200)</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="F49" s="26" t="n">
+        <x:f>COUNT('Data'!$H$334:$H$349,'Data'!$H$1185:$H$1200)</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="G49" s="27" t="n">
+        <x:f>IF(F49=0,"—",SUM('Data'!$H$334:$H$349,'Data'!$H$1185:$H$1200)/F49/100)</x:f>
+        <x:v>0.8780000000000001</x:v>
+      </x:c>
+      <x:c r="H49" s="27" t="n">
+        <x:f>IF(E49=0,"—",SUM('Data'!$H$334:$H$349,'Data'!$H$1185:$H$1200)/E49/100)</x:f>
+        <x:v>0.8780000000000001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="23" customHeight="1">
+      <x:c r="B50" s="22" t="str">
+        <x:v>Csv</x:v>
+      </x:c>
+      <x:c r="C50" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D50" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E50" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$334:$D$349,'Data'!$D$1185:$D$1200)</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="F50" s="26" t="n">
+        <x:f>COUNT('Data'!$K$334:$K$349,'Data'!$K$1185:$K$1200)</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="G50" s="27" t="n">
+        <x:f>IF(F50=0,"—",SUM('Data'!$K$334:$K$349,'Data'!$K$1185:$K$1200)/F50/100)</x:f>
+        <x:v>0.79791875</x:v>
+      </x:c>
+      <x:c r="H50" s="27" t="n">
+        <x:f>IF(E50=0,"—",SUM('Data'!$K$334:$K$349,'Data'!$K$1185:$K$1200)/E50/100)</x:f>
+        <x:v>0.79791875</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="23" customHeight="1">
+      <x:c r="B51" s="22" t="str">
+        <x:v>Csv</x:v>
+      </x:c>
+      <x:c r="C51" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D51" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E51" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$334:$D$349)</x:f>
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="F51" s="26" t="n">
+        <x:f>COUNT('Data'!$H$334:$H$349)</x:f>
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G51" s="27" t="n">
+        <x:f>IF(F51=0,"—",SUM('Data'!$H$334:$H$349)/F51/100)</x:f>
+        <x:v>0.8780000000000001</x:v>
+      </x:c>
+      <x:c r="H51" s="27" t="n">
+        <x:f>IF(E51=0,"—",SUM('Data'!$H$334:$H$349)/E51/100)</x:f>
+        <x:v>0.8780000000000001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="23" customHeight="1">
+      <x:c r="B52" s="22" t="str">
+        <x:v>Csv</x:v>
+      </x:c>
+      <x:c r="C52" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D52" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E52" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$334:$D$349)</x:f>
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="F52" s="26" t="n">
+        <x:f>COUNT('Data'!$K$334:$K$349)</x:f>
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G52" s="27" t="n">
+        <x:f>IF(F52=0,"—",SUM('Data'!$K$334:$K$349)/F52/100)</x:f>
+        <x:v>0.79791875</x:v>
+      </x:c>
+      <x:c r="H52" s="27" t="n">
+        <x:f>IF(E52=0,"—",SUM('Data'!$K$334:$K$349)/E52/100)</x:f>
+        <x:v>0.79791875</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="23" customHeight="1">
+      <x:c r="B53" s="22" t="str">
+        <x:v>Csv</x:v>
+      </x:c>
+      <x:c r="C53" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D53" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E53" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$1185:$D$1200)</x:f>
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="F53" s="26" t="n">
+        <x:f>COUNT('Data'!$H$1185:$H$1200)</x:f>
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G53" s="27" t="n">
+        <x:f>IF(F53=0,"—",SUM('Data'!$H$1185:$H$1200)/F53/100)</x:f>
+        <x:v>0.8780000000000001</x:v>
+      </x:c>
+      <x:c r="H53" s="27" t="n">
+        <x:f>IF(E53=0,"—",SUM('Data'!$H$1185:$H$1200)/E53/100)</x:f>
+        <x:v>0.8780000000000001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="23" customHeight="1">
+      <x:c r="B54" s="22" t="str">
+        <x:v>Csv</x:v>
+      </x:c>
+      <x:c r="C54" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D54" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E54" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$1185:$D$1200)</x:f>
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="F54" s="26" t="n">
+        <x:f>COUNT('Data'!$K$1185:$K$1200)</x:f>
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G54" s="27" t="n">
+        <x:f>IF(F54=0,"—",SUM('Data'!$K$1185:$K$1200)/F54/100)</x:f>
+        <x:v>0.79791875</x:v>
+      </x:c>
+      <x:c r="H54" s="27" t="n">
+        <x:f>IF(E54=0,"—",SUM('Data'!$K$1185:$K$1200)/E54/100)</x:f>
+        <x:v>0.79791875</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="23" customHeight="1">
+      <x:c r="B55" s="22" t="str">
+        <x:v>Gson</x:v>
+      </x:c>
+      <x:c r="C55" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D55" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E55" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$350:$D$366,'Data'!$D$1201:$D$1217)</x:f>
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="F55" s="26" t="n">
+        <x:f>COUNT('Data'!$H$350:$H$366,'Data'!$H$1201:$H$1217)</x:f>
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="G55" s="27" t="n">
+        <x:f>IF(F55=0,"—",SUM('Data'!$H$350:$H$366,'Data'!$H$1201:$H$1217)/F55/100)</x:f>
+        <x:v>0.42284705882352946</x:v>
+      </x:c>
+      <x:c r="H55" s="27" t="n">
+        <x:f>IF(E55=0,"—",SUM('Data'!$H$350:$H$366,'Data'!$H$1201:$H$1217)/E55/100)</x:f>
+        <x:v>0.42284705882352946</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="23" customHeight="1">
+      <x:c r="B56" s="22" t="str">
+        <x:v>Gson</x:v>
+      </x:c>
+      <x:c r="C56" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D56" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E56" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$350:$D$366,'Data'!$D$1201:$D$1217)</x:f>
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="F56" s="26" t="n">
+        <x:f>COUNT('Data'!$K$350:$K$366,'Data'!$K$1201:$K$1217)</x:f>
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="G56" s="27" t="n">
+        <x:f>IF(F56=0,"—",SUM('Data'!$K$350:$K$366,'Data'!$K$1201:$K$1217)/F56/100)</x:f>
+        <x:v>0.3498117647058824</x:v>
+      </x:c>
+      <x:c r="H56" s="27" t="n">
+        <x:f>IF(E56=0,"—",SUM('Data'!$K$350:$K$366,'Data'!$K$1201:$K$1217)/E56/100)</x:f>
+        <x:v>0.3498117647058824</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="23" customHeight="1">
+      <x:c r="B57" s="22" t="str">
+        <x:v>Gson</x:v>
+      </x:c>
+      <x:c r="C57" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D57" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E57" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$350:$D$366)</x:f>
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="F57" s="26" t="n">
+        <x:f>COUNT('Data'!$H$350:$H$366)</x:f>
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="G57" s="27" t="n">
+        <x:f>IF(F57=0,"—",SUM('Data'!$H$350:$H$366)/F57/100)</x:f>
+        <x:v>0.42284705882352946</x:v>
+      </x:c>
+      <x:c r="H57" s="27" t="n">
+        <x:f>IF(E57=0,"—",SUM('Data'!$H$350:$H$366)/E57/100)</x:f>
+        <x:v>0.42284705882352946</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="23" customHeight="1">
+      <x:c r="B58" s="22" t="str">
+        <x:v>Gson</x:v>
+      </x:c>
+      <x:c r="C58" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D58" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E58" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$350:$D$366)</x:f>
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="F58" s="26" t="n">
+        <x:f>COUNT('Data'!$K$350:$K$366)</x:f>
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="G58" s="27" t="n">
+        <x:f>IF(F58=0,"—",SUM('Data'!$K$350:$K$366)/F58/100)</x:f>
+        <x:v>0.3498117647058824</x:v>
+      </x:c>
+      <x:c r="H58" s="27" t="n">
+        <x:f>IF(E58=0,"—",SUM('Data'!$K$350:$K$366)/E58/100)</x:f>
+        <x:v>0.3498117647058824</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="23" customHeight="1">
+      <x:c r="B59" s="22" t="str">
+        <x:v>Gson</x:v>
+      </x:c>
+      <x:c r="C59" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D59" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E59" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$1201:$D$1217)</x:f>
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="F59" s="26" t="n">
+        <x:f>COUNT('Data'!$H$1201:$H$1217)</x:f>
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="G59" s="27" t="n">
+        <x:f>IF(F59=0,"—",SUM('Data'!$H$1201:$H$1217)/F59/100)</x:f>
+        <x:v>0.42284705882352946</x:v>
+      </x:c>
+      <x:c r="H59" s="27" t="n">
+        <x:f>IF(E59=0,"—",SUM('Data'!$H$1201:$H$1217)/E59/100)</x:f>
+        <x:v>0.42284705882352946</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="23" customHeight="1">
+      <x:c r="B60" s="22" t="str">
+        <x:v>Gson</x:v>
+      </x:c>
+      <x:c r="C60" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D60" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E60" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$1201:$D$1217)</x:f>
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="F60" s="26" t="n">
+        <x:f>COUNT('Data'!$K$1201:$K$1217)</x:f>
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="G60" s="27" t="n">
+        <x:f>IF(F60=0,"—",SUM('Data'!$K$1201:$K$1217)/F60/100)</x:f>
+        <x:v>0.3498117647058824</x:v>
+      </x:c>
+      <x:c r="H60" s="27" t="n">
+        <x:f>IF(E60=0,"—",SUM('Data'!$K$1201:$K$1217)/E60/100)</x:f>
+        <x:v>0.3498117647058824</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="23" customHeight="1">
+      <x:c r="B61" s="22" t="str">
+        <x:v>JacksonCore</x:v>
+      </x:c>
+      <x:c r="C61" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D61" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E61" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$367:$D$390,'Data'!$D$1218:$D$1241)</x:f>
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="F61" s="26" t="n">
+        <x:f>COUNT('Data'!$H$367:$H$390,'Data'!$H$1218:$H$1241)</x:f>
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="G61" s="27" t="n">
+        <x:f>IF(F61=0,"—",SUM('Data'!$H$367:$H$390,'Data'!$H$1218:$H$1241)/F61/100)</x:f>
+        <x:v>0.5649958333333334</x:v>
+      </x:c>
+      <x:c r="H61" s="27" t="n">
+        <x:f>IF(E61=0,"—",SUM('Data'!$H$367:$H$390,'Data'!$H$1218:$H$1241)/E61/100)</x:f>
+        <x:v>0.5649958333333334</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="23" customHeight="1">
+      <x:c r="B62" s="22" t="str">
+        <x:v>JacksonCore</x:v>
+      </x:c>
+      <x:c r="C62" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D62" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E62" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$367:$D$390,'Data'!$D$1218:$D$1241)</x:f>
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="F62" s="26" t="n">
+        <x:f>COUNT('Data'!$K$367:$K$390,'Data'!$K$1218:$K$1241)</x:f>
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="G62" s="27" t="n">
+        <x:f>IF(F62=0,"—",SUM('Data'!$K$367:$K$390,'Data'!$K$1218:$K$1241)/F62/100)</x:f>
+        <x:v>0.4709125</x:v>
+      </x:c>
+      <x:c r="H62" s="27" t="n">
+        <x:f>IF(E62=0,"—",SUM('Data'!$K$367:$K$390,'Data'!$K$1218:$K$1241)/E62/100)</x:f>
+        <x:v>0.4709125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="23" customHeight="1">
+      <x:c r="B63" s="22" t="str">
+        <x:v>JacksonCore</x:v>
+      </x:c>
+      <x:c r="C63" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D63" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E63" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$367:$D$390)</x:f>
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="F63" s="26" t="n">
+        <x:f>COUNT('Data'!$H$367:$H$390)</x:f>
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="G63" s="27" t="n">
+        <x:f>IF(F63=0,"—",SUM('Data'!$H$367:$H$390)/F63/100)</x:f>
+        <x:v>0.5649958333333334</x:v>
+      </x:c>
+      <x:c r="H63" s="27" t="n">
+        <x:f>IF(E63=0,"—",SUM('Data'!$H$367:$H$390)/E63/100)</x:f>
+        <x:v>0.5649958333333334</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="23" customHeight="1">
+      <x:c r="B64" s="22" t="str">
+        <x:v>JacksonCore</x:v>
+      </x:c>
+      <x:c r="C64" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D64" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E64" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$367:$D$390)</x:f>
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="F64" s="26" t="n">
+        <x:f>COUNT('Data'!$K$367:$K$390)</x:f>
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="G64" s="27" t="n">
+        <x:f>IF(F64=0,"—",SUM('Data'!$K$367:$K$390)/F64/100)</x:f>
+        <x:v>0.4709125</x:v>
+      </x:c>
+      <x:c r="H64" s="27" t="n">
+        <x:f>IF(E64=0,"—",SUM('Data'!$K$367:$K$390)/E64/100)</x:f>
+        <x:v>0.4709125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="23" customHeight="1">
+      <x:c r="B65" s="22" t="str">
+        <x:v>JacksonCore</x:v>
+      </x:c>
+      <x:c r="C65" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D65" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E65" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$1218:$D$1241)</x:f>
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="F65" s="26" t="n">
+        <x:f>COUNT('Data'!$H$1218:$H$1241)</x:f>
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="G65" s="27" t="n">
+        <x:f>IF(F65=0,"—",SUM('Data'!$H$1218:$H$1241)/F65/100)</x:f>
+        <x:v>0.5649958333333334</x:v>
+      </x:c>
+      <x:c r="H65" s="27" t="n">
+        <x:f>IF(E65=0,"—",SUM('Data'!$H$1218:$H$1241)/E65/100)</x:f>
+        <x:v>0.5649958333333334</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="23" customHeight="1">
+      <x:c r="B66" s="22" t="str">
+        <x:v>JacksonCore</x:v>
+      </x:c>
+      <x:c r="C66" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D66" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E66" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$1218:$D$1241)</x:f>
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="F66" s="26" t="n">
+        <x:f>COUNT('Data'!$K$1218:$K$1241)</x:f>
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="G66" s="27" t="n">
+        <x:f>IF(F66=0,"—",SUM('Data'!$K$1218:$K$1241)/F66/100)</x:f>
+        <x:v>0.4709125</x:v>
+      </x:c>
+      <x:c r="H66" s="27" t="n">
+        <x:f>IF(E66=0,"—",SUM('Data'!$K$1218:$K$1241)/E66/100)</x:f>
+        <x:v>0.4709125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="23" customHeight="1">
+      <x:c r="B67" s="22" t="str">
+        <x:v>JacksonDatabind</x:v>
+      </x:c>
+      <x:c r="C67" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D67" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E67" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$391:$D$500,'Data'!$D$1242:$D$1351)</x:f>
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="F67" s="26" t="n">
+        <x:f>COUNT('Data'!$H$391:$H$500,'Data'!$H$1242:$H$1351)</x:f>
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="G67" s="27" t="n">
+        <x:f>IF(F67=0,"—",SUM('Data'!$H$391:$H$500,'Data'!$H$1242:$H$1351)/F67/100)</x:f>
+        <x:v>0.590779090909091</x:v>
+      </x:c>
+      <x:c r="H67" s="27" t="n">
+        <x:f>IF(E67=0,"—",SUM('Data'!$H$391:$H$500,'Data'!$H$1242:$H$1351)/E67/100)</x:f>
+        <x:v>0.590779090909091</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="23" customHeight="1">
+      <x:c r="B68" s="22" t="str">
+        <x:v>JacksonDatabind</x:v>
+      </x:c>
+      <x:c r="C68" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D68" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E68" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$391:$D$500,'Data'!$D$1242:$D$1351)</x:f>
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="F68" s="26" t="n">
+        <x:f>COUNT('Data'!$K$391:$K$500,'Data'!$K$1242:$K$1351)</x:f>
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="G68" s="27" t="n">
+        <x:f>IF(F68=0,"—",SUM('Data'!$K$391:$K$500,'Data'!$K$1242:$K$1351)/F68/100)</x:f>
+        <x:v>0.47467636363636373</x:v>
+      </x:c>
+      <x:c r="H68" s="27" t="n">
+        <x:f>IF(E68=0,"—",SUM('Data'!$K$391:$K$500,'Data'!$K$1242:$K$1351)/E68/100)</x:f>
+        <x:v>0.47467636363636373</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="23" customHeight="1">
+      <x:c r="B69" s="22" t="str">
+        <x:v>JacksonDatabind</x:v>
+      </x:c>
+      <x:c r="C69" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D69" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E69" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$391:$D$500)</x:f>
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="F69" s="26" t="n">
+        <x:f>COUNT('Data'!$H$391:$H$500)</x:f>
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="G69" s="27" t="n">
+        <x:f>IF(F69=0,"—",SUM('Data'!$H$391:$H$500)/F69/100)</x:f>
+        <x:v>0.590779090909091</x:v>
+      </x:c>
+      <x:c r="H69" s="27" t="n">
+        <x:f>IF(E69=0,"—",SUM('Data'!$H$391:$H$500)/E69/100)</x:f>
+        <x:v>0.590779090909091</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="23" customHeight="1">
+      <x:c r="B70" s="22" t="str">
+        <x:v>JacksonDatabind</x:v>
+      </x:c>
+      <x:c r="C70" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D70" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E70" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$391:$D$500)</x:f>
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="F70" s="26" t="n">
+        <x:f>COUNT('Data'!$K$391:$K$500)</x:f>
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="G70" s="27" t="n">
+        <x:f>IF(F70=0,"—",SUM('Data'!$K$391:$K$500)/F70/100)</x:f>
+        <x:v>0.47467636363636373</x:v>
+      </x:c>
+      <x:c r="H70" s="27" t="n">
+        <x:f>IF(E70=0,"—",SUM('Data'!$K$391:$K$500)/E70/100)</x:f>
+        <x:v>0.47467636363636373</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="23" customHeight="1">
+      <x:c r="B71" s="22" t="str">
+        <x:v>JacksonDatabind</x:v>
+      </x:c>
+      <x:c r="C71" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D71" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E71" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$1242:$D$1351)</x:f>
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="F71" s="26" t="n">
+        <x:f>COUNT('Data'!$H$1242:$H$1351)</x:f>
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="G71" s="27" t="n">
+        <x:f>IF(F71=0,"—",SUM('Data'!$H$1242:$H$1351)/F71/100)</x:f>
+        <x:v>0.590779090909091</x:v>
+      </x:c>
+      <x:c r="H71" s="27" t="n">
+        <x:f>IF(E71=0,"—",SUM('Data'!$H$1242:$H$1351)/E71/100)</x:f>
+        <x:v>0.590779090909091</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="23" customHeight="1">
+      <x:c r="B72" s="22" t="str">
+        <x:v>JacksonDatabind</x:v>
+      </x:c>
+      <x:c r="C72" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D72" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E72" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$1242:$D$1351)</x:f>
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="F72" s="26" t="n">
+        <x:f>COUNT('Data'!$K$1242:$K$1351)</x:f>
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="G72" s="27" t="n">
+        <x:f>IF(F72=0,"—",SUM('Data'!$K$1242:$K$1351)/F72/100)</x:f>
+        <x:v>0.47467636363636373</x:v>
+      </x:c>
+      <x:c r="H72" s="27" t="n">
+        <x:f>IF(E72=0,"—",SUM('Data'!$K$1242:$K$1351)/E72/100)</x:f>
+        <x:v>0.47467636363636373</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="23" customHeight="1">
+      <x:c r="B73" s="22" t="str">
+        <x:v>JacksonXml</x:v>
+      </x:c>
+      <x:c r="C73" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D73" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E73" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$501:$D$506,'Data'!$D$1352:$D$1357)</x:f>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F73" s="26" t="n">
+        <x:f>COUNT('Data'!$H$501:$H$506,'Data'!$H$1352:$H$1357)</x:f>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="G73" s="27" t="n">
+        <x:f>IF(F73=0,"—",SUM('Data'!$H$501:$H$506,'Data'!$H$1352:$H$1357)/F73/100)</x:f>
+        <x:v>0.3019166666666667</x:v>
+      </x:c>
+      <x:c r="H73" s="27" t="n">
+        <x:f>IF(E73=0,"—",SUM('Data'!$H$501:$H$506,'Data'!$H$1352:$H$1357)/E73/100)</x:f>
+        <x:v>0.3019166666666667</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="23" customHeight="1">
+      <x:c r="B74" s="22" t="str">
+        <x:v>JacksonXml</x:v>
+      </x:c>
+      <x:c r="C74" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D74" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E74" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$501:$D$506,'Data'!$D$1352:$D$1357)</x:f>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F74" s="26" t="n">
+        <x:f>COUNT('Data'!$K$501:$K$506,'Data'!$K$1352:$K$1357)</x:f>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="G74" s="27" t="n">
+        <x:f>IF(F74=0,"—",SUM('Data'!$K$501:$K$506,'Data'!$K$1352:$K$1357)/F74/100)</x:f>
+        <x:v>0.24133333333333337</x:v>
+      </x:c>
+      <x:c r="H74" s="27" t="n">
+        <x:f>IF(E74=0,"—",SUM('Data'!$K$501:$K$506,'Data'!$K$1352:$K$1357)/E74/100)</x:f>
+        <x:v>0.24133333333333337</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="23" customHeight="1">
+      <x:c r="B75" s="22" t="str">
+        <x:v>JacksonXml</x:v>
+      </x:c>
+      <x:c r="C75" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D75" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E75" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$501:$D$506)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F75" s="26" t="n">
+        <x:f>COUNT('Data'!$H$501:$H$506)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G75" s="27" t="n">
+        <x:f>IF(F75=0,"—",SUM('Data'!$H$501:$H$506)/F75/100)</x:f>
+        <x:v>0.3019166666666667</x:v>
+      </x:c>
+      <x:c r="H75" s="27" t="n">
+        <x:f>IF(E75=0,"—",SUM('Data'!$H$501:$H$506)/E75/100)</x:f>
+        <x:v>0.3019166666666667</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="23" customHeight="1">
+      <x:c r="B76" s="22" t="str">
+        <x:v>JacksonXml</x:v>
+      </x:c>
+      <x:c r="C76" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D76" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E76" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$501:$D$506)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F76" s="26" t="n">
+        <x:f>COUNT('Data'!$K$501:$K$506)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G76" s="27" t="n">
+        <x:f>IF(F76=0,"—",SUM('Data'!$K$501:$K$506)/F76/100)</x:f>
+        <x:v>0.24133333333333337</x:v>
+      </x:c>
+      <x:c r="H76" s="27" t="n">
+        <x:f>IF(E76=0,"—",SUM('Data'!$K$501:$K$506)/E76/100)</x:f>
+        <x:v>0.24133333333333337</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="23" customHeight="1">
+      <x:c r="B77" s="22" t="str">
+        <x:v>JacksonXml</x:v>
+      </x:c>
+      <x:c r="C77" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D77" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E77" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$1352:$D$1357)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F77" s="26" t="n">
+        <x:f>COUNT('Data'!$H$1352:$H$1357)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G77" s="27" t="n">
+        <x:f>IF(F77=0,"—",SUM('Data'!$H$1352:$H$1357)/F77/100)</x:f>
+        <x:v>0.3019166666666667</x:v>
+      </x:c>
+      <x:c r="H77" s="27" t="n">
+        <x:f>IF(E77=0,"—",SUM('Data'!$H$1352:$H$1357)/E77/100)</x:f>
+        <x:v>0.3019166666666667</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="23" customHeight="1">
+      <x:c r="B78" s="22" t="str">
+        <x:v>JacksonXml</x:v>
+      </x:c>
+      <x:c r="C78" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D78" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E78" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$1352:$D$1357)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F78" s="26" t="n">
+        <x:f>COUNT('Data'!$K$1352:$K$1357)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G78" s="27" t="n">
+        <x:f>IF(F78=0,"—",SUM('Data'!$K$1352:$K$1357)/F78/100)</x:f>
+        <x:v>0.24133333333333337</x:v>
+      </x:c>
+      <x:c r="H78" s="27" t="n">
+        <x:f>IF(E78=0,"—",SUM('Data'!$K$1352:$K$1357)/E78/100)</x:f>
+        <x:v>0.24133333333333337</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="23" customHeight="1">
+      <x:c r="B79" s="22" t="str">
+        <x:v>Jsoup</x:v>
+      </x:c>
+      <x:c r="C79" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D79" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E79" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$507:$D$599,'Data'!$D$1358:$D$1450)</x:f>
+        <x:v>186</x:v>
+      </x:c>
+      <x:c r="F79" s="26" t="n">
+        <x:f>COUNT('Data'!$H$507:$H$599,'Data'!$H$1358:$H$1450)</x:f>
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="G79" s="27" t="n">
+        <x:f>IF(F79=0,"—",SUM('Data'!$H$507:$H$599,'Data'!$H$1358:$H$1450)/F79/100)</x:f>
+        <x:v>0.6899055555555554</x:v>
+      </x:c>
+      <x:c r="H79" s="27" t="n">
+        <x:f>IF(E79=0,"—",SUM('Data'!$H$507:$H$599,'Data'!$H$1358:$H$1450)/E79/100)</x:f>
+        <x:v>0.6676505376344086</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="23" customHeight="1">
+      <x:c r="B80" s="22" t="str">
+        <x:v>Jsoup</x:v>
+      </x:c>
+      <x:c r="C80" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D80" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E80" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$507:$D$599,'Data'!$D$1358:$D$1450)</x:f>
+        <x:v>186</x:v>
+      </x:c>
+      <x:c r="F80" s="26" t="n">
+        <x:f>COUNT('Data'!$K$507:$K$599,'Data'!$K$1358:$K$1450)</x:f>
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="G80" s="27" t="n">
+        <x:f>IF(F80=0,"—",SUM('Data'!$K$507:$K$599,'Data'!$K$1358:$K$1450)/F80/100)</x:f>
+        <x:v>0.6155322222222221</x:v>
+      </x:c>
+      <x:c r="H80" s="27" t="n">
+        <x:f>IF(E80=0,"—",SUM('Data'!$K$507:$K$599,'Data'!$K$1358:$K$1450)/E80/100)</x:f>
+        <x:v>0.5956763440860214</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="23" customHeight="1">
+      <x:c r="B81" s="22" t="str">
+        <x:v>Jsoup</x:v>
+      </x:c>
+      <x:c r="C81" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D81" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E81" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$507:$D$599)</x:f>
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="F81" s="26" t="n">
+        <x:f>COUNT('Data'!$H$507:$H$599)</x:f>
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="G81" s="27" t="n">
+        <x:f>IF(F81=0,"—",SUM('Data'!$H$507:$H$599)/F81/100)</x:f>
+        <x:v>0.6899055555555554</x:v>
+      </x:c>
+      <x:c r="H81" s="27" t="n">
+        <x:f>IF(E81=0,"—",SUM('Data'!$H$507:$H$599)/E81/100)</x:f>
+        <x:v>0.6676505376344086</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="23" customHeight="1">
+      <x:c r="B82" s="22" t="str">
+        <x:v>Jsoup</x:v>
+      </x:c>
+      <x:c r="C82" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D82" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E82" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$507:$D$599)</x:f>
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="F82" s="26" t="n">
+        <x:f>COUNT('Data'!$K$507:$K$599)</x:f>
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="G82" s="27" t="n">
+        <x:f>IF(F82=0,"—",SUM('Data'!$K$507:$K$599)/F82/100)</x:f>
+        <x:v>0.6155322222222221</x:v>
+      </x:c>
+      <x:c r="H82" s="27" t="n">
+        <x:f>IF(E82=0,"—",SUM('Data'!$K$507:$K$599)/E82/100)</x:f>
+        <x:v>0.5956763440860214</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="23" customHeight="1">
+      <x:c r="B83" s="22" t="str">
+        <x:v>Jsoup</x:v>
+      </x:c>
+      <x:c r="C83" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D83" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E83" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$1358:$D$1450)</x:f>
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="F83" s="26" t="n">
+        <x:f>COUNT('Data'!$H$1358:$H$1450)</x:f>
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="G83" s="27" t="n">
+        <x:f>IF(F83=0,"—",SUM('Data'!$H$1358:$H$1450)/F83/100)</x:f>
+        <x:v>0.6899055555555554</x:v>
+      </x:c>
+      <x:c r="H83" s="27" t="n">
+        <x:f>IF(E83=0,"—",SUM('Data'!$H$1358:$H$1450)/E83/100)</x:f>
+        <x:v>0.6676505376344086</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="23" customHeight="1">
+      <x:c r="B84" s="22" t="str">
+        <x:v>Jsoup</x:v>
+      </x:c>
+      <x:c r="C84" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D84" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E84" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$1358:$D$1450)</x:f>
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="F84" s="26" t="n">
+        <x:f>COUNT('Data'!$K$1358:$K$1450)</x:f>
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="G84" s="27" t="n">
+        <x:f>IF(F84=0,"—",SUM('Data'!$K$1358:$K$1450)/F84/100)</x:f>
+        <x:v>0.6155322222222221</x:v>
+      </x:c>
+      <x:c r="H84" s="27" t="n">
+        <x:f>IF(E84=0,"—",SUM('Data'!$K$1358:$K$1450)/E84/100)</x:f>
+        <x:v>0.5956763440860214</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="23" customHeight="1">
+      <x:c r="B85" s="22" t="str">
+        <x:v>JxPath</x:v>
+      </x:c>
+      <x:c r="C85" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D85" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E85" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$600:$D$621,'Data'!$D$1451:$D$1472)</x:f>
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="F85" s="26" t="n">
+        <x:f>COUNT('Data'!$H$600:$H$621,'Data'!$H$1451:$H$1472)</x:f>
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="G85" s="27" t="n">
+        <x:f>IF(F85=0,"—",SUM('Data'!$H$600:$H$621,'Data'!$H$1451:$H$1472)/F85/100)</x:f>
+        <x:v>0.783490909090909</x:v>
+      </x:c>
+      <x:c r="H85" s="27" t="n">
+        <x:f>IF(E85=0,"—",SUM('Data'!$H$600:$H$621,'Data'!$H$1451:$H$1472)/E85/100)</x:f>
+        <x:v>0.783490909090909</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="23" customHeight="1">
+      <x:c r="B86" s="22" t="str">
+        <x:v>JxPath</x:v>
+      </x:c>
+      <x:c r="C86" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D86" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E86" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$600:$D$621,'Data'!$D$1451:$D$1472)</x:f>
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="F86" s="26" t="n">
+        <x:f>COUNT('Data'!$K$600:$K$621,'Data'!$K$1451:$K$1472)</x:f>
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="G86" s="27" t="n">
+        <x:f>IF(F86=0,"—",SUM('Data'!$K$600:$K$621,'Data'!$K$1451:$K$1472)/F86/100)</x:f>
+        <x:v>0.7114909090909091</x:v>
+      </x:c>
+      <x:c r="H86" s="27" t="n">
+        <x:f>IF(E86=0,"—",SUM('Data'!$K$600:$K$621,'Data'!$K$1451:$K$1472)/E86/100)</x:f>
+        <x:v>0.7114909090909091</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="23" customHeight="1">
+      <x:c r="B87" s="22" t="str">
+        <x:v>JxPath</x:v>
+      </x:c>
+      <x:c r="C87" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D87" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E87" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$600:$D$621)</x:f>
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="F87" s="26" t="n">
+        <x:f>COUNT('Data'!$H$600:$H$621)</x:f>
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G87" s="27" t="n">
+        <x:f>IF(F87=0,"—",SUM('Data'!$H$600:$H$621)/F87/100)</x:f>
+        <x:v>0.783490909090909</x:v>
+      </x:c>
+      <x:c r="H87" s="27" t="n">
+        <x:f>IF(E87=0,"—",SUM('Data'!$H$600:$H$621)/E87/100)</x:f>
+        <x:v>0.783490909090909</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="23" customHeight="1">
+      <x:c r="B88" s="22" t="str">
+        <x:v>JxPath</x:v>
+      </x:c>
+      <x:c r="C88" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D88" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E88" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$600:$D$621)</x:f>
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="F88" s="26" t="n">
+        <x:f>COUNT('Data'!$K$600:$K$621)</x:f>
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G88" s="27" t="n">
+        <x:f>IF(F88=0,"—",SUM('Data'!$K$600:$K$621)/F88/100)</x:f>
+        <x:v>0.7114909090909091</x:v>
+      </x:c>
+      <x:c r="H88" s="27" t="n">
+        <x:f>IF(E88=0,"—",SUM('Data'!$K$600:$K$621)/E88/100)</x:f>
+        <x:v>0.7114909090909091</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="23" customHeight="1">
+      <x:c r="B89" s="22" t="str">
+        <x:v>JxPath</x:v>
+      </x:c>
+      <x:c r="C89" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D89" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E89" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$1451:$D$1472)</x:f>
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="F89" s="26" t="n">
+        <x:f>COUNT('Data'!$H$1451:$H$1472)</x:f>
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G89" s="27" t="n">
+        <x:f>IF(F89=0,"—",SUM('Data'!$H$1451:$H$1472)/F89/100)</x:f>
+        <x:v>0.783490909090909</x:v>
+      </x:c>
+      <x:c r="H89" s="27" t="n">
+        <x:f>IF(E89=0,"—",SUM('Data'!$H$1451:$H$1472)/E89/100)</x:f>
+        <x:v>0.783490909090909</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="23" customHeight="1">
+      <x:c r="B90" s="22" t="str">
+        <x:v>JxPath</x:v>
+      </x:c>
+      <x:c r="C90" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D90" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E90" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$1451:$D$1472)</x:f>
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="F90" s="26" t="n">
+        <x:f>COUNT('Data'!$K$1451:$K$1472)</x:f>
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G90" s="27" t="n">
+        <x:f>IF(F90=0,"—",SUM('Data'!$K$1451:$K$1472)/F90/100)</x:f>
+        <x:v>0.7114909090909091</x:v>
+      </x:c>
+      <x:c r="H90" s="27" t="n">
+        <x:f>IF(E90=0,"—",SUM('Data'!$K$1451:$K$1472)/E90/100)</x:f>
+        <x:v>0.7114909090909091</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="23" customHeight="1">
+      <x:c r="B91" s="22" t="str">
+        <x:v>Lang</x:v>
+      </x:c>
+      <x:c r="C91" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D91" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E91" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$622:$D$682,'Data'!$D$1473:$D$1533)</x:f>
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="F91" s="26" t="n">
+        <x:f>COUNT('Data'!$H$622:$H$682,'Data'!$H$1473:$H$1533)</x:f>
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="G91" s="27" t="n">
+        <x:f>IF(F91=0,"—",SUM('Data'!$H$622:$H$682,'Data'!$H$1473:$H$1533)/F91/100)</x:f>
+        <x:v>0.8432409836065574</x:v>
+      </x:c>
+      <x:c r="H91" s="27" t="n">
+        <x:f>IF(E91=0,"—",SUM('Data'!$H$622:$H$682,'Data'!$H$1473:$H$1533)/E91/100)</x:f>
+        <x:v>0.8432409836065574</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="23" customHeight="1">
+      <x:c r="B92" s="22" t="str">
+        <x:v>Lang</x:v>
+      </x:c>
+      <x:c r="C92" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D92" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E92" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$622:$D$682,'Data'!$D$1473:$D$1533)</x:f>
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="F92" s="26" t="n">
+        <x:f>COUNT('Data'!$K$622:$K$682,'Data'!$K$1473:$K$1533)</x:f>
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="G92" s="27" t="n">
+        <x:f>IF(F92=0,"—",SUM('Data'!$K$622:$K$682,'Data'!$K$1473:$K$1533)/F92/100)</x:f>
+        <x:v>0.7932803278688525</x:v>
+      </x:c>
+      <x:c r="H92" s="27" t="n">
+        <x:f>IF(E92=0,"—",SUM('Data'!$K$622:$K$682,'Data'!$K$1473:$K$1533)/E92/100)</x:f>
+        <x:v>0.7932803278688525</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="23" customHeight="1">
+      <x:c r="B93" s="22" t="str">
+        <x:v>Lang</x:v>
+      </x:c>
+      <x:c r="C93" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D93" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E93" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$622:$D$682)</x:f>
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="F93" s="26" t="n">
+        <x:f>COUNT('Data'!$H$622:$H$682)</x:f>
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="G93" s="27" t="n">
+        <x:f>IF(F93=0,"—",SUM('Data'!$H$622:$H$682)/F93/100)</x:f>
+        <x:v>0.8432409836065574</x:v>
+      </x:c>
+      <x:c r="H93" s="27" t="n">
+        <x:f>IF(E93=0,"—",SUM('Data'!$H$622:$H$682)/E93/100)</x:f>
+        <x:v>0.8432409836065574</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="23" customHeight="1">
+      <x:c r="B94" s="22" t="str">
+        <x:v>Lang</x:v>
+      </x:c>
+      <x:c r="C94" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D94" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E94" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$622:$D$682)</x:f>
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="F94" s="26" t="n">
+        <x:f>COUNT('Data'!$K$622:$K$682)</x:f>
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="G94" s="27" t="n">
+        <x:f>IF(F94=0,"—",SUM('Data'!$K$622:$K$682)/F94/100)</x:f>
+        <x:v>0.7932803278688525</x:v>
+      </x:c>
+      <x:c r="H94" s="27" t="n">
+        <x:f>IF(E94=0,"—",SUM('Data'!$K$622:$K$682)/E94/100)</x:f>
+        <x:v>0.7932803278688525</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="23" customHeight="1">
+      <x:c r="B95" s="22" t="str">
+        <x:v>Lang</x:v>
+      </x:c>
+      <x:c r="C95" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D95" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E95" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$1473:$D$1533)</x:f>
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="F95" s="26" t="n">
+        <x:f>COUNT('Data'!$H$1473:$H$1533)</x:f>
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="G95" s="27" t="n">
+        <x:f>IF(F95=0,"—",SUM('Data'!$H$1473:$H$1533)/F95/100)</x:f>
+        <x:v>0.8432409836065574</x:v>
+      </x:c>
+      <x:c r="H95" s="27" t="n">
+        <x:f>IF(E95=0,"—",SUM('Data'!$H$1473:$H$1533)/E95/100)</x:f>
+        <x:v>0.8432409836065574</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="23" customHeight="1">
+      <x:c r="B96" s="22" t="str">
+        <x:v>Lang</x:v>
+      </x:c>
+      <x:c r="C96" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D96" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E96" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$1473:$D$1533)</x:f>
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="F96" s="26" t="n">
+        <x:f>COUNT('Data'!$K$1473:$K$1533)</x:f>
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="G96" s="27" t="n">
+        <x:f>IF(F96=0,"—",SUM('Data'!$K$1473:$K$1533)/F96/100)</x:f>
+        <x:v>0.7932803278688525</x:v>
+      </x:c>
+      <x:c r="H96" s="27" t="n">
+        <x:f>IF(E96=0,"—",SUM('Data'!$K$1473:$K$1533)/E96/100)</x:f>
+        <x:v>0.7932803278688525</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97" ht="23" customHeight="1">
+      <x:c r="B97" s="22" t="str">
+        <x:v>Math</x:v>
+      </x:c>
+      <x:c r="C97" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D97" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E97" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$683:$D$788,'Data'!$D$1534:$D$1639)</x:f>
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="F97" s="26" t="n">
+        <x:f>COUNT('Data'!$H$683:$H$788,'Data'!$H$1534:$H$1639)</x:f>
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="G97" s="27" t="n">
+        <x:f>IF(F97=0,"—",SUM('Data'!$H$683:$H$788,'Data'!$H$1534:$H$1639)/F97/100)</x:f>
+        <x:v>0.8430990196078432</x:v>
+      </x:c>
+      <x:c r="H97" s="27" t="n">
+        <x:f>IF(E97=0,"—",SUM('Data'!$H$683:$H$788,'Data'!$H$1534:$H$1639)/E97/100)</x:f>
+        <x:v>0.811283962264151</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="23" customHeight="1">
+      <x:c r="B98" s="22" t="str">
+        <x:v>Math</x:v>
+      </x:c>
+      <x:c r="C98" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D98" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E98" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$683:$D$788,'Data'!$D$1534:$D$1639)</x:f>
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="F98" s="26" t="n">
+        <x:f>COUNT('Data'!$K$683:$K$788,'Data'!$K$1534:$K$1639)</x:f>
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="G98" s="27" t="n">
+        <x:f>IF(F98=0,"—",SUM('Data'!$K$683:$K$788,'Data'!$K$1534:$K$1639)/F98/100)</x:f>
+        <x:v>0.8131431372549018</x:v>
+      </x:c>
+      <x:c r="H98" s="27" t="n">
+        <x:f>IF(E98=0,"—",SUM('Data'!$K$683:$K$788,'Data'!$K$1534:$K$1639)/E98/100)</x:f>
+        <x:v>0.7824584905660374</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="23" customHeight="1">
+      <x:c r="B99" s="22" t="str">
+        <x:v>Math</x:v>
+      </x:c>
+      <x:c r="C99" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D99" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E99" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$683:$D$788)</x:f>
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="F99" s="26" t="n">
+        <x:f>COUNT('Data'!$H$683:$H$788)</x:f>
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="G99" s="27" t="n">
+        <x:f>IF(F99=0,"—",SUM('Data'!$H$683:$H$788)/F99/100)</x:f>
+        <x:v>0.842484693877551</x:v>
+      </x:c>
+      <x:c r="H99" s="27" t="n">
+        <x:f>IF(E99=0,"—",SUM('Data'!$H$683:$H$788)/E99/100)</x:f>
+        <x:v>0.7789009433962262</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="23" customHeight="1">
+      <x:c r="B100" s="22" t="str">
+        <x:v>Math</x:v>
+      </x:c>
+      <x:c r="C100" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D100" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E100" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$683:$D$788)</x:f>
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="F100" s="26" t="n">
+        <x:f>COUNT('Data'!$K$683:$K$788)</x:f>
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="G100" s="27" t="n">
+        <x:f>IF(F100=0,"—",SUM('Data'!$K$683:$K$788)/F100/100)</x:f>
+        <x:v>0.8119683673469386</x:v>
+      </x:c>
+      <x:c r="H100" s="27" t="n">
+        <x:f>IF(E100=0,"—",SUM('Data'!$K$683:$K$788)/E100/100)</x:f>
+        <x:v>0.7506877358490565</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="23" customHeight="1">
+      <x:c r="B101" s="22" t="str">
+        <x:v>Math</x:v>
+      </x:c>
+      <x:c r="C101" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D101" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E101" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$1534:$D$1639)</x:f>
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="F101" s="26" t="n">
+        <x:f>COUNT('Data'!$H$1534:$H$1639)</x:f>
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="G101" s="27" t="n">
+        <x:f>IF(F101=0,"—",SUM('Data'!$H$1534:$H$1639)/F101/100)</x:f>
+        <x:v>0.8436669811320755</x:v>
+      </x:c>
+      <x:c r="H101" s="27" t="n">
+        <x:f>IF(E101=0,"—",SUM('Data'!$H$1534:$H$1639)/E101/100)</x:f>
+        <x:v>0.8436669811320755</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102" ht="23" customHeight="1">
+      <x:c r="B102" s="22" t="str">
+        <x:v>Math</x:v>
+      </x:c>
+      <x:c r="C102" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D102" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E102" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$1534:$D$1639)</x:f>
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="F102" s="26" t="n">
+        <x:f>COUNT('Data'!$K$1534:$K$1639)</x:f>
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="G102" s="27" t="n">
+        <x:f>IF(F102=0,"—",SUM('Data'!$K$1534:$K$1639)/F102/100)</x:f>
+        <x:v>0.8142292452830187</x:v>
+      </x:c>
+      <x:c r="H102" s="27" t="n">
+        <x:f>IF(E102=0,"—",SUM('Data'!$K$1534:$K$1639)/E102/100)</x:f>
+        <x:v>0.8142292452830187</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103" ht="23" customHeight="1">
+      <x:c r="B103" s="22" t="str">
+        <x:v>Mockito</x:v>
+      </x:c>
+      <x:c r="C103" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D103" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E103" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$789:$D$826,'Data'!$D$1640:$D$1677)</x:f>
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="F103" s="26" t="n">
+        <x:f>COUNT('Data'!$H$789:$H$826,'Data'!$H$1640:$H$1677)</x:f>
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="G103" s="27" t="n">
+        <x:f>IF(F103=0,"—",SUM('Data'!$H$789:$H$826,'Data'!$H$1640:$H$1677)/F103/100)</x:f>
+        <x:v>0.5254394736842105</x:v>
+      </x:c>
+      <x:c r="H103" s="27" t="n">
+        <x:f>IF(E103=0,"—",SUM('Data'!$H$789:$H$826,'Data'!$H$1640:$H$1677)/E103/100)</x:f>
+        <x:v>0.5254394736842105</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="23" customHeight="1">
+      <x:c r="B104" s="22" t="str">
+        <x:v>Mockito</x:v>
+      </x:c>
+      <x:c r="C104" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D104" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E104" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$789:$D$826,'Data'!$D$1640:$D$1677)</x:f>
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="F104" s="26" t="n">
+        <x:f>COUNT('Data'!$K$789:$K$826,'Data'!$K$1640:$K$1677)</x:f>
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="G104" s="27" t="n">
+        <x:f>IF(F104=0,"—",SUM('Data'!$K$789:$K$826,'Data'!$K$1640:$K$1677)/F104/100)</x:f>
+        <x:v>0.36180285714285715</x:v>
+      </x:c>
+      <x:c r="H104" s="27" t="n">
+        <x:f>IF(E104=0,"—",SUM('Data'!$K$789:$K$826,'Data'!$K$1640:$K$1677)/E104/100)</x:f>
+        <x:v>0.3332394736842106</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105" ht="23" customHeight="1">
+      <x:c r="B105" s="22" t="str">
+        <x:v>Mockito</x:v>
+      </x:c>
+      <x:c r="C105" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D105" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E105" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$789:$D$826)</x:f>
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="F105" s="26" t="n">
+        <x:f>COUNT('Data'!$H$789:$H$826)</x:f>
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="G105" s="27" t="n">
+        <x:f>IF(F105=0,"—",SUM('Data'!$H$789:$H$826)/F105/100)</x:f>
+        <x:v>0.5254394736842105</x:v>
+      </x:c>
+      <x:c r="H105" s="27" t="n">
+        <x:f>IF(E105=0,"—",SUM('Data'!$H$789:$H$826)/E105/100)</x:f>
+        <x:v>0.5254394736842105</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="23" customHeight="1">
+      <x:c r="B106" s="22" t="str">
+        <x:v>Mockito</x:v>
+      </x:c>
+      <x:c r="C106" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D106" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E106" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$789:$D$826)</x:f>
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="F106" s="26" t="n">
+        <x:f>COUNT('Data'!$K$789:$K$826)</x:f>
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="G106" s="27" t="n">
+        <x:f>IF(F106=0,"—",SUM('Data'!$K$789:$K$826)/F106/100)</x:f>
+        <x:v>0.36180285714285715</x:v>
+      </x:c>
+      <x:c r="H106" s="27" t="n">
+        <x:f>IF(E106=0,"—",SUM('Data'!$K$789:$K$826)/E106/100)</x:f>
+        <x:v>0.3332394736842106</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="23" customHeight="1">
+      <x:c r="B107" s="22" t="str">
+        <x:v>Mockito</x:v>
+      </x:c>
+      <x:c r="C107" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D107" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E107" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$1640:$D$1677)</x:f>
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="F107" s="26" t="n">
+        <x:f>COUNT('Data'!$H$1640:$H$1677)</x:f>
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="G107" s="27" t="n">
+        <x:f>IF(F107=0,"—",SUM('Data'!$H$1640:$H$1677)/F107/100)</x:f>
+        <x:v>0.5254394736842105</x:v>
+      </x:c>
+      <x:c r="H107" s="27" t="n">
+        <x:f>IF(E107=0,"—",SUM('Data'!$H$1640:$H$1677)/E107/100)</x:f>
+        <x:v>0.5254394736842105</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="23" customHeight="1">
+      <x:c r="B108" s="22" t="str">
+        <x:v>Mockito</x:v>
+      </x:c>
+      <x:c r="C108" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D108" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E108" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$1640:$D$1677)</x:f>
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="F108" s="26" t="n">
+        <x:f>COUNT('Data'!$K$1640:$K$1677)</x:f>
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="G108" s="27" t="n">
+        <x:f>IF(F108=0,"—",SUM('Data'!$K$1640:$K$1677)/F108/100)</x:f>
+        <x:v>0.36180285714285715</x:v>
+      </x:c>
+      <x:c r="H108" s="27" t="n">
+        <x:f>IF(E108=0,"—",SUM('Data'!$K$1640:$K$1677)/E108/100)</x:f>
+        <x:v>0.3332394736842106</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="23" customHeight="1">
+      <x:c r="B109" s="22" t="str">
+        <x:v>Time</x:v>
+      </x:c>
+      <x:c r="C109" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D109" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E109" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$827:$D$852,'Data'!$D$1678:$D$1703)</x:f>
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="F109" s="26" t="n">
+        <x:f>COUNT('Data'!$H$827:$H$852,'Data'!$H$1678:$H$1703)</x:f>
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="G109" s="27" t="n">
+        <x:f>IF(F109=0,"—",SUM('Data'!$H$827:$H$852,'Data'!$H$1678:$H$1703)/F109/100)</x:f>
+        <x:v>0.868726923076923</x:v>
+      </x:c>
+      <x:c r="H109" s="27" t="n">
+        <x:f>IF(E109=0,"—",SUM('Data'!$H$827:$H$852,'Data'!$H$1678:$H$1703)/E109/100)</x:f>
+        <x:v>0.868726923076923</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="23" customHeight="1">
+      <x:c r="B110" s="22" t="str">
+        <x:v>Time</x:v>
+      </x:c>
+      <x:c r="C110" s="22" t="str">
+        <x:v>All rounds</x:v>
+      </x:c>
+      <x:c r="D110" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E110" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$827:$D$852,'Data'!$D$1678:$D$1703)</x:f>
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="F110" s="26" t="n">
+        <x:f>COUNT('Data'!$K$827:$K$852,'Data'!$K$1678:$K$1703)</x:f>
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="G110" s="27" t="n">
+        <x:f>IF(F110=0,"—",SUM('Data'!$K$827:$K$852,'Data'!$K$1678:$K$1703)/F110/100)</x:f>
+        <x:v>0.7958961538461539</x:v>
+      </x:c>
+      <x:c r="H110" s="27" t="n">
+        <x:f>IF(E110=0,"—",SUM('Data'!$K$827:$K$852,'Data'!$K$1678:$K$1703)/E110/100)</x:f>
+        <x:v>0.7958961538461539</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111" ht="23" customHeight="1">
+      <x:c r="B111" s="22" t="str">
+        <x:v>Time</x:v>
+      </x:c>
+      <x:c r="C111" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D111" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E111" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$827:$D$852)</x:f>
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="F111" s="26" t="n">
+        <x:f>COUNT('Data'!$H$827:$H$852)</x:f>
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="G111" s="27" t="n">
+        <x:f>IF(F111=0,"—",SUM('Data'!$H$827:$H$852)/F111/100)</x:f>
+        <x:v>0.868726923076923</x:v>
+      </x:c>
+      <x:c r="H111" s="27" t="n">
+        <x:f>IF(E111=0,"—",SUM('Data'!$H$827:$H$852)/E111/100)</x:f>
+        <x:v>0.868726923076923</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112" ht="23" customHeight="1">
+      <x:c r="B112" s="22" t="str">
+        <x:v>Time</x:v>
+      </x:c>
+      <x:c r="C112" s="22" t="str">
+        <x:v>Round1</x:v>
+      </x:c>
+      <x:c r="D112" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E112" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$827:$D$852)</x:f>
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="F112" s="26" t="n">
+        <x:f>COUNT('Data'!$K$827:$K$852)</x:f>
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="G112" s="27" t="n">
+        <x:f>IF(F112=0,"—",SUM('Data'!$K$827:$K$852)/F112/100)</x:f>
+        <x:v>0.7958961538461539</x:v>
+      </x:c>
+      <x:c r="H112" s="27" t="n">
+        <x:f>IF(E112=0,"—",SUM('Data'!$K$827:$K$852)/E112/100)</x:f>
+        <x:v>0.7958961538461539</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113" ht="23" customHeight="1">
+      <x:c r="B113" s="22" t="str">
+        <x:v>Time</x:v>
+      </x:c>
+      <x:c r="C113" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D113" s="22" t="str">
+        <x:v>Line</x:v>
+      </x:c>
+      <x:c r="E113" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$1678:$D$1703)</x:f>
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="F113" s="26" t="n">
+        <x:f>COUNT('Data'!$H$1678:$H$1703)</x:f>
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="G113" s="27" t="n">
+        <x:f>IF(F113=0,"—",SUM('Data'!$H$1678:$H$1703)/F113/100)</x:f>
+        <x:v>0.868726923076923</x:v>
+      </x:c>
+      <x:c r="H113" s="27" t="n">
+        <x:f>IF(E113=0,"—",SUM('Data'!$H$1678:$H$1703)/E113/100)</x:f>
+        <x:v>0.868726923076923</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114" ht="23" customHeight="1">
+      <x:c r="B114" s="22" t="str">
+        <x:v>Time</x:v>
+      </x:c>
+      <x:c r="C114" s="22" t="str">
+        <x:v>Round2</x:v>
+      </x:c>
+      <x:c r="D114" s="22" t="str">
+        <x:v>Condition</x:v>
+      </x:c>
+      <x:c r="E114" s="26" t="n">
+        <x:f>COUNTA('Data'!$D$1678:$D$1703)</x:f>
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="F114" s="26" t="n">
+        <x:f>COUNT('Data'!$K$1678:$K$1703)</x:f>
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="G114" s="27" t="n">
+        <x:f>IF(F114=0,"—",SUM('Data'!$K$1678:$K$1703)/F114/100)</x:f>
+        <x:v>0.7958961538461539</x:v>
+      </x:c>
+      <x:c r="H114" s="27" t="n">
+        <x:f>IF(E114=0,"—",SUM('Data'!$K$1678:$K$1703)/E114/100)</x:f>
+        <x:v>0.7958961538461539</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="B3:H3"/>
+    <x:mergeCell ref="B4:H4"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>